<commit_message>
CCD-8295: Removing spaces and updating xls
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jen/IdeaProjects/test-defs-jen/ccd-test-definitions/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954FA031-EF13-2646-8FAB-9E530A767D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3EAACDF-5AA6-2D45-BDC1-BFD2E3A4E2B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" firstSheet="15" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" firstSheet="8" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SearchInputFields" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16208" uniqueCount="1559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16209" uniqueCount="1558">
   <si>
     <t>SearchInputFields</t>
   </si>
@@ -4154,9 +4154,6 @@
   </si>
   <si>
     <t>Staff User Fields</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#ARGUMENT(CATEGORY-LEGAL-OPS,CATEGORY-ADMIN,REGION-1235) </t>
   </si>
   <si>
     <t>AllOrgPoliciesPage</t>
@@ -28778,7 +28775,7 @@
         <v>1220</v>
       </c>
       <c r="P257" s="2" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="258" spans="1:16">
@@ -49597,7 +49594,7 @@
         <v>1</v>
       </c>
       <c r="O311" t="s">
-        <v>1368</v>
+        <v>1557</v>
       </c>
       <c r="P311" t="s">
         <v>714</v>
@@ -49632,7 +49629,7 @@
         <v>1</v>
       </c>
       <c r="O312" t="s">
-        <v>1368</v>
+        <v>1557</v>
       </c>
       <c r="P312" t="s">
         <v>714</v>
@@ -50266,7 +50263,7 @@
         <v>1300</v>
       </c>
       <c r="H332" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="I332" t="s">
         <v>1296</v>
@@ -50298,7 +50295,7 @@
         <v>1300</v>
       </c>
       <c r="H333" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="I333" t="s">
         <v>1296</v>
@@ -50330,7 +50327,7 @@
         <v>1300</v>
       </c>
       <c r="H334" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="I334" t="s">
         <v>1296</v>
@@ -51538,7 +51535,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>1370</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -51563,10 +51560,10 @@
         <v>729</v>
       </c>
       <c r="C4" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
       <c r="D4" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -51577,10 +51574,10 @@
         <v>729</v>
       </c>
       <c r="C5" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
       <c r="D5" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -51591,10 +51588,10 @@
         <v>1238</v>
       </c>
       <c r="C6" t="s">
+        <v>1371</v>
+      </c>
+      <c r="D6" t="s">
         <v>1372</v>
-      </c>
-      <c r="D6" t="s">
-        <v>1373</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -51605,10 +51602,10 @@
         <v>1249</v>
       </c>
       <c r="C7" t="s">
+        <v>1373</v>
+      </c>
+      <c r="D7" t="s">
         <v>1374</v>
-      </c>
-      <c r="D7" t="s">
-        <v>1375</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -51619,10 +51616,10 @@
         <v>1238</v>
       </c>
       <c r="C8" t="s">
+        <v>1371</v>
+      </c>
+      <c r="D8" t="s">
         <v>1372</v>
-      </c>
-      <c r="D8" t="s">
-        <v>1373</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -51633,10 +51630,10 @@
         <v>1249</v>
       </c>
       <c r="C9" t="s">
+        <v>1373</v>
+      </c>
+      <c r="D9" t="s">
         <v>1374</v>
-      </c>
-      <c r="D9" t="s">
-        <v>1375</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -51647,10 +51644,10 @@
         <v>1249</v>
       </c>
       <c r="C10" t="s">
+        <v>1373</v>
+      </c>
+      <c r="D10" t="s">
         <v>1374</v>
-      </c>
-      <c r="D10" t="s">
-        <v>1375</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -51661,10 +51658,10 @@
         <v>1238</v>
       </c>
       <c r="C11" t="s">
+        <v>1371</v>
+      </c>
+      <c r="D11" t="s">
         <v>1372</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1373</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -51675,10 +51672,10 @@
         <v>1249</v>
       </c>
       <c r="C12" t="s">
+        <v>1373</v>
+      </c>
+      <c r="D12" t="s">
         <v>1374</v>
-      </c>
-      <c r="D12" t="s">
-        <v>1375</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -51689,10 +51686,10 @@
         <v>747</v>
       </c>
       <c r="C13" t="s">
+        <v>1375</v>
+      </c>
+      <c r="D13" t="s">
         <v>1376</v>
-      </c>
-      <c r="D13" t="s">
-        <v>1377</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -51703,10 +51700,10 @@
         <v>826</v>
       </c>
       <c r="C14" t="s">
+        <v>1377</v>
+      </c>
+      <c r="D14" t="s">
         <v>1378</v>
-      </c>
-      <c r="D14" t="s">
-        <v>1379</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -51717,10 +51714,10 @@
         <v>1258</v>
       </c>
       <c r="C15" t="s">
+        <v>1379</v>
+      </c>
+      <c r="D15" t="s">
         <v>1380</v>
-      </c>
-      <c r="D15" t="s">
-        <v>1381</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -51731,10 +51728,10 @@
         <v>1261</v>
       </c>
       <c r="C16" t="s">
+        <v>1381</v>
+      </c>
+      <c r="D16" t="s">
         <v>1382</v>
-      </c>
-      <c r="D16" t="s">
-        <v>1383</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -51745,10 +51742,10 @@
         <v>1264</v>
       </c>
       <c r="C17" t="s">
+        <v>1383</v>
+      </c>
+      <c r="D17" t="s">
         <v>1384</v>
-      </c>
-      <c r="D17" t="s">
-        <v>1385</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -51759,10 +51756,10 @@
         <v>1258</v>
       </c>
       <c r="C18" t="s">
+        <v>1379</v>
+      </c>
+      <c r="D18" t="s">
         <v>1380</v>
-      </c>
-      <c r="D18" t="s">
-        <v>1381</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -51773,10 +51770,10 @@
         <v>1261</v>
       </c>
       <c r="C19" t="s">
+        <v>1381</v>
+      </c>
+      <c r="D19" t="s">
         <v>1382</v>
-      </c>
-      <c r="D19" t="s">
-        <v>1383</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -51787,10 +51784,10 @@
         <v>1264</v>
       </c>
       <c r="C20" t="s">
+        <v>1383</v>
+      </c>
+      <c r="D20" t="s">
         <v>1384</v>
-      </c>
-      <c r="D20" t="s">
-        <v>1385</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -51801,10 +51798,10 @@
         <v>1258</v>
       </c>
       <c r="C21" t="s">
+        <v>1379</v>
+      </c>
+      <c r="D21" t="s">
         <v>1380</v>
-      </c>
-      <c r="D21" t="s">
-        <v>1381</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -51815,10 +51812,10 @@
         <v>1261</v>
       </c>
       <c r="C22" t="s">
+        <v>1381</v>
+      </c>
+      <c r="D22" t="s">
         <v>1382</v>
-      </c>
-      <c r="D22" t="s">
-        <v>1383</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -51829,10 +51826,10 @@
         <v>1264</v>
       </c>
       <c r="C23" t="s">
+        <v>1383</v>
+      </c>
+      <c r="D23" t="s">
         <v>1384</v>
-      </c>
-      <c r="D23" t="s">
-        <v>1385</v>
       </c>
     </row>
   </sheetData>
@@ -51847,7 +51844,7 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -51867,22 +51864,22 @@
         <v>646</v>
       </c>
       <c r="F3" t="s">
+        <v>1386</v>
+      </c>
+      <c r="G3" t="s">
         <v>1387</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>1388</v>
-      </c>
-      <c r="H3" t="s">
-        <v>1389</v>
       </c>
       <c r="I3" t="s">
         <v>187</v>
       </c>
       <c r="J3" t="s">
+        <v>1389</v>
+      </c>
+      <c r="K3" t="s">
         <v>1390</v>
-      </c>
-      <c r="K3" t="s">
-        <v>1391</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -51893,16 +51890,16 @@
         <v>114</v>
       </c>
       <c r="D4" t="s">
+        <v>1391</v>
+      </c>
+      <c r="E4" t="s">
         <v>1392</v>
-      </c>
-      <c r="E4" t="s">
-        <v>1393</v>
       </c>
       <c r="F4" t="s">
         <v>177</v>
       </c>
       <c r="G4" t="s">
-        <v>1394</v>
+        <v>1393</v>
       </c>
       <c r="I4" t="s">
         <v>218</v>
@@ -51916,10 +51913,10 @@
         <v>56</v>
       </c>
       <c r="D5" t="s">
+        <v>1394</v>
+      </c>
+      <c r="E5" t="s">
         <v>1395</v>
-      </c>
-      <c r="E5" t="s">
-        <v>1396</v>
       </c>
       <c r="F5" t="s">
         <v>177</v>
@@ -51936,10 +51933,10 @@
         <v>110</v>
       </c>
       <c r="D6" t="s">
+        <v>1396</v>
+      </c>
+      <c r="E6" t="s">
         <v>1397</v>
-      </c>
-      <c r="E6" t="s">
-        <v>1398</v>
       </c>
       <c r="F6" t="s">
         <v>177</v>
@@ -51956,10 +51953,10 @@
         <v>60</v>
       </c>
       <c r="D7" t="s">
+        <v>1398</v>
+      </c>
+      <c r="E7" t="s">
         <v>1399</v>
-      </c>
-      <c r="E7" t="s">
-        <v>1400</v>
       </c>
       <c r="F7" t="s">
         <v>177</v>
@@ -51976,10 +51973,10 @@
         <v>93</v>
       </c>
       <c r="D8" t="s">
+        <v>1400</v>
+      </c>
+      <c r="E8" t="s">
         <v>1401</v>
-      </c>
-      <c r="E8" t="s">
-        <v>1402</v>
       </c>
       <c r="F8" t="s">
         <v>177</v>
@@ -51996,10 +51993,10 @@
         <v>78</v>
       </c>
       <c r="D9" t="s">
+        <v>1402</v>
+      </c>
+      <c r="E9" t="s">
         <v>1403</v>
-      </c>
-      <c r="E9" t="s">
-        <v>1404</v>
       </c>
       <c r="F9" t="s">
         <v>177</v>
@@ -52016,10 +52013,10 @@
         <v>105</v>
       </c>
       <c r="D10" t="s">
+        <v>1404</v>
+      </c>
+      <c r="E10" t="s">
         <v>1405</v>
-      </c>
-      <c r="E10" t="s">
-        <v>1406</v>
       </c>
       <c r="F10" t="s">
         <v>177</v>
@@ -52036,10 +52033,10 @@
         <v>83</v>
       </c>
       <c r="D11" t="s">
+        <v>1406</v>
+      </c>
+      <c r="E11" t="s">
         <v>1407</v>
-      </c>
-      <c r="E11" t="s">
-        <v>1408</v>
       </c>
       <c r="F11" t="s">
         <v>177</v>
@@ -52056,10 +52053,10 @@
         <v>113</v>
       </c>
       <c r="D12" t="s">
+        <v>1408</v>
+      </c>
+      <c r="E12" t="s">
         <v>1409</v>
-      </c>
-      <c r="E12" t="s">
-        <v>1410</v>
       </c>
       <c r="F12" t="s">
         <v>177</v>
@@ -52076,10 +52073,10 @@
         <v>156</v>
       </c>
       <c r="D13" t="s">
+        <v>1410</v>
+      </c>
+      <c r="E13" t="s">
         <v>1411</v>
-      </c>
-      <c r="E13" t="s">
-        <v>1412</v>
       </c>
       <c r="F13" t="s">
         <v>177</v>
@@ -52096,10 +52093,10 @@
         <v>157</v>
       </c>
       <c r="D14" t="s">
+        <v>1412</v>
+      </c>
+      <c r="E14" t="s">
         <v>1413</v>
-      </c>
-      <c r="E14" t="s">
-        <v>1414</v>
       </c>
       <c r="F14" t="s">
         <v>177</v>
@@ -52116,10 +52113,10 @@
         <v>109</v>
       </c>
       <c r="D15" t="s">
+        <v>1414</v>
+      </c>
+      <c r="E15" t="s">
         <v>1415</v>
-      </c>
-      <c r="E15" t="s">
-        <v>1416</v>
       </c>
       <c r="F15" t="s">
         <v>177</v>
@@ -52136,16 +52133,16 @@
         <v>9</v>
       </c>
       <c r="D16" t="s">
+        <v>1416</v>
+      </c>
+      <c r="E16" t="s">
         <v>1417</v>
-      </c>
-      <c r="E16" t="s">
-        <v>1418</v>
       </c>
       <c r="F16" t="s">
         <v>177</v>
       </c>
       <c r="G16" t="s">
-        <v>1394</v>
+        <v>1393</v>
       </c>
       <c r="I16" t="s">
         <v>218</v>
@@ -52159,10 +52156,10 @@
         <v>103</v>
       </c>
       <c r="D17" t="s">
+        <v>1418</v>
+      </c>
+      <c r="E17" t="s">
         <v>1419</v>
-      </c>
-      <c r="E17" t="s">
-        <v>1420</v>
       </c>
       <c r="F17" t="s">
         <v>177</v>
@@ -52179,10 +52176,10 @@
         <v>81</v>
       </c>
       <c r="D18" t="s">
+        <v>1420</v>
+      </c>
+      <c r="E18" t="s">
         <v>1421</v>
-      </c>
-      <c r="E18" t="s">
-        <v>1422</v>
       </c>
       <c r="F18" t="s">
         <v>177</v>
@@ -52199,10 +52196,10 @@
         <v>79</v>
       </c>
       <c r="D19" t="s">
+        <v>1422</v>
+      </c>
+      <c r="E19" t="s">
         <v>1423</v>
-      </c>
-      <c r="E19" t="s">
-        <v>1424</v>
       </c>
       <c r="F19" t="s">
         <v>177</v>
@@ -52219,10 +52216,10 @@
         <v>150</v>
       </c>
       <c r="D20" t="s">
+        <v>1424</v>
+      </c>
+      <c r="E20" t="s">
         <v>1425</v>
-      </c>
-      <c r="E20" t="s">
-        <v>1426</v>
       </c>
       <c r="F20" t="s">
         <v>177</v>
@@ -52239,10 +52236,10 @@
         <v>151</v>
       </c>
       <c r="D21" t="s">
+        <v>1426</v>
+      </c>
+      <c r="E21" t="s">
         <v>1427</v>
-      </c>
-      <c r="E21" t="s">
-        <v>1428</v>
       </c>
       <c r="F21" t="s">
         <v>177</v>
@@ -52259,10 +52256,10 @@
         <v>140</v>
       </c>
       <c r="D22" t="s">
+        <v>1428</v>
+      </c>
+      <c r="E22" t="s">
         <v>1429</v>
-      </c>
-      <c r="E22" t="s">
-        <v>1430</v>
       </c>
       <c r="F22" t="s">
         <v>177</v>
@@ -52279,10 +52276,10 @@
         <v>54</v>
       </c>
       <c r="D23" t="s">
+        <v>1430</v>
+      </c>
+      <c r="E23" t="s">
         <v>1431</v>
-      </c>
-      <c r="E23" t="s">
-        <v>1432</v>
       </c>
       <c r="F23" t="s">
         <v>177</v>
@@ -52299,10 +52296,10 @@
         <v>59</v>
       </c>
       <c r="D24" t="s">
+        <v>1432</v>
+      </c>
+      <c r="E24" t="s">
         <v>1433</v>
-      </c>
-      <c r="E24" t="s">
-        <v>1434</v>
       </c>
       <c r="F24" t="s">
         <v>177</v>
@@ -52319,10 +52316,10 @@
         <v>106</v>
       </c>
       <c r="D25" t="s">
+        <v>1434</v>
+      </c>
+      <c r="E25" t="s">
         <v>1435</v>
-      </c>
-      <c r="E25" t="s">
-        <v>1436</v>
       </c>
       <c r="F25" t="s">
         <v>177</v>
@@ -52339,10 +52336,10 @@
         <v>152</v>
       </c>
       <c r="D26" t="s">
+        <v>1436</v>
+      </c>
+      <c r="E26" t="s">
         <v>1437</v>
-      </c>
-      <c r="E26" t="s">
-        <v>1438</v>
       </c>
       <c r="F26" t="s">
         <v>177</v>
@@ -52359,10 +52356,10 @@
         <v>139</v>
       </c>
       <c r="D27" t="s">
+        <v>1438</v>
+      </c>
+      <c r="E27" t="s">
         <v>1439</v>
-      </c>
-      <c r="E27" t="s">
-        <v>1440</v>
       </c>
       <c r="F27" t="s">
         <v>177</v>
@@ -52379,10 +52376,10 @@
         <v>138</v>
       </c>
       <c r="D28" t="s">
+        <v>1440</v>
+      </c>
+      <c r="E28" t="s">
         <v>1441</v>
-      </c>
-      <c r="E28" t="s">
-        <v>1442</v>
       </c>
       <c r="F28" t="s">
         <v>177</v>
@@ -52399,10 +52396,10 @@
         <v>153</v>
       </c>
       <c r="D29" t="s">
+        <v>1442</v>
+      </c>
+      <c r="E29" t="s">
         <v>1443</v>
-      </c>
-      <c r="E29" t="s">
-        <v>1444</v>
       </c>
       <c r="F29" t="s">
         <v>177</v>
@@ -52419,10 +52416,10 @@
         <v>76</v>
       </c>
       <c r="D30" t="s">
+        <v>1444</v>
+      </c>
+      <c r="E30" t="s">
         <v>1445</v>
-      </c>
-      <c r="E30" t="s">
-        <v>1446</v>
       </c>
       <c r="F30" t="s">
         <v>177</v>
@@ -52442,7 +52439,7 @@
         <v>94</v>
       </c>
       <c r="E31" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
       <c r="F31" t="s">
         <v>177</v>
@@ -52462,7 +52459,7 @@
         <v>55</v>
       </c>
       <c r="E32" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
       <c r="F32" t="s">
         <v>177</v>
@@ -52482,7 +52479,7 @@
         <v>111</v>
       </c>
       <c r="E33" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
       <c r="F33" t="s">
         <v>177</v>
@@ -52502,7 +52499,7 @@
         <v>49</v>
       </c>
       <c r="E34" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
       <c r="F34" t="s">
         <v>177</v>
@@ -52522,7 +52519,7 @@
         <v>33</v>
       </c>
       <c r="E35" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="F35" t="s">
         <v>177</v>
@@ -52542,7 +52539,7 @@
         <v>162</v>
       </c>
       <c r="E36" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="F36" t="s">
         <v>177</v>
@@ -52562,7 +52559,7 @@
         <v>96</v>
       </c>
       <c r="E37" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="F37" t="s">
         <v>177</v>
@@ -52582,7 +52579,7 @@
         <v>80</v>
       </c>
       <c r="E38" t="s">
-        <v>1450</v>
+        <v>1449</v>
       </c>
       <c r="F38" t="s">
         <v>177</v>
@@ -52602,7 +52599,7 @@
         <v>161</v>
       </c>
       <c r="E39" t="s">
-        <v>1451</v>
+        <v>1450</v>
       </c>
       <c r="F39" t="s">
         <v>177</v>
@@ -52622,7 +52619,7 @@
         <v>149</v>
       </c>
       <c r="E40" t="s">
-        <v>1452</v>
+        <v>1451</v>
       </c>
       <c r="F40" t="s">
         <v>177</v>
@@ -52642,7 +52639,7 @@
         <v>77</v>
       </c>
       <c r="E41" t="s">
-        <v>1453</v>
+        <v>1452</v>
       </c>
       <c r="F41" t="s">
         <v>177</v>
@@ -52662,7 +52659,7 @@
         <v>112</v>
       </c>
       <c r="E42" t="s">
-        <v>1454</v>
+        <v>1453</v>
       </c>
       <c r="F42" t="s">
         <v>177</v>
@@ -52682,7 +52679,7 @@
         <v>108</v>
       </c>
       <c r="E43" t="s">
-        <v>1455</v>
+        <v>1454</v>
       </c>
       <c r="F43" t="s">
         <v>177</v>
@@ -52702,7 +52699,7 @@
         <v>50</v>
       </c>
       <c r="E44" t="s">
-        <v>1456</v>
+        <v>1455</v>
       </c>
       <c r="F44" t="s">
         <v>177</v>
@@ -52722,7 +52719,7 @@
         <v>154</v>
       </c>
       <c r="E45" t="s">
-        <v>1457</v>
+        <v>1456</v>
       </c>
       <c r="F45" t="s">
         <v>177</v>
@@ -52742,7 +52739,7 @@
         <v>155</v>
       </c>
       <c r="E46" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
       <c r="F46" t="s">
         <v>177</v>
@@ -52751,7 +52748,7 @@
         <v>218</v>
       </c>
       <c r="J46" t="s">
-        <v>1459</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -52765,7 +52762,7 @@
         <v>104</v>
       </c>
       <c r="E47" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
       <c r="F47" t="s">
         <v>177</v>
@@ -52785,7 +52782,7 @@
         <v>42</v>
       </c>
       <c r="E48" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
       <c r="F48" t="s">
         <v>177</v>
@@ -52805,7 +52802,7 @@
         <v>53</v>
       </c>
       <c r="E49" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
       <c r="F49" t="s">
         <v>177</v>
@@ -52825,7 +52822,7 @@
         <v>159</v>
       </c>
       <c r="E50" t="s">
-        <v>1460</v>
+        <v>1459</v>
       </c>
       <c r="F50" t="s">
         <v>177</v>
@@ -52845,7 +52842,7 @@
         <v>75</v>
       </c>
       <c r="E51" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
       <c r="F51" t="s">
         <v>177</v>
@@ -52865,7 +52862,7 @@
         <v>46</v>
       </c>
       <c r="E52" t="s">
-        <v>1462</v>
+        <v>1461</v>
       </c>
       <c r="F52" t="s">
         <v>177</v>
@@ -52885,7 +52882,7 @@
         <v>160</v>
       </c>
       <c r="E53" t="s">
-        <v>1463</v>
+        <v>1462</v>
       </c>
       <c r="F53" t="s">
         <v>177</v>
@@ -52905,7 +52902,7 @@
         <v>98</v>
       </c>
       <c r="E54" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="F54" t="s">
         <v>177</v>
@@ -52925,7 +52922,7 @@
         <v>63</v>
       </c>
       <c r="E55" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="F55" t="s">
         <v>177</v>
@@ -52972,7 +52969,7 @@
         <v>7</v>
       </c>
       <c r="H3" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -52986,7 +52983,7 @@
         <v>721</v>
       </c>
       <c r="E4" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -53003,7 +53000,7 @@
         <v>722</v>
       </c>
       <c r="E5" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="G5">
         <v>2</v>
@@ -53020,7 +53017,7 @@
         <v>723</v>
       </c>
       <c r="E6" t="s">
-        <v>1469</v>
+        <v>1468</v>
       </c>
       <c r="G6">
         <v>3</v>
@@ -53037,7 +53034,7 @@
         <v>178</v>
       </c>
       <c r="E7" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -53054,7 +53051,7 @@
         <v>178</v>
       </c>
       <c r="E8" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -53071,7 +53068,7 @@
         <v>725</v>
       </c>
       <c r="E9" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G9">
         <v>1</v>
@@ -53088,7 +53085,7 @@
         <v>178</v>
       </c>
       <c r="E10" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -53105,7 +53102,7 @@
         <v>725</v>
       </c>
       <c r="E11" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G11">
         <v>1</v>
@@ -53122,7 +53119,7 @@
         <v>178</v>
       </c>
       <c r="E12" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G12">
         <v>1</v>
@@ -53139,7 +53136,7 @@
         <v>725</v>
       </c>
       <c r="E13" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G13">
         <v>1</v>
@@ -53156,7 +53153,7 @@
         <v>178</v>
       </c>
       <c r="E14" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -53173,7 +53170,7 @@
         <v>178</v>
       </c>
       <c r="E15" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -53190,7 +53187,7 @@
         <v>725</v>
       </c>
       <c r="E16" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -53207,7 +53204,7 @@
         <v>178</v>
       </c>
       <c r="E17" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -53224,7 +53221,7 @@
         <v>178</v>
       </c>
       <c r="E18" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -53241,7 +53238,7 @@
         <v>725</v>
       </c>
       <c r="E19" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -53258,7 +53255,7 @@
         <v>178</v>
       </c>
       <c r="E20" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G20">
         <v>1</v>
@@ -53275,7 +53272,7 @@
         <v>733</v>
       </c>
       <c r="E21" t="s">
-        <v>1472</v>
+        <v>1471</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -53292,7 +53289,7 @@
         <v>178</v>
       </c>
       <c r="E22" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -53309,7 +53306,7 @@
         <v>725</v>
       </c>
       <c r="E23" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -53326,7 +53323,7 @@
         <v>734</v>
       </c>
       <c r="E24" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -53343,7 +53340,7 @@
         <v>178</v>
       </c>
       <c r="E25" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -53360,7 +53357,7 @@
         <v>178</v>
       </c>
       <c r="E26" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G26">
         <v>1</v>
@@ -53377,7 +53374,7 @@
         <v>725</v>
       </c>
       <c r="E27" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G27">
         <v>2</v>
@@ -53394,7 +53391,7 @@
         <v>178</v>
       </c>
       <c r="E28" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G28">
         <v>1</v>
@@ -53411,7 +53408,7 @@
         <v>725</v>
       </c>
       <c r="E29" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G29">
         <v>1</v>
@@ -53428,7 +53425,7 @@
         <v>178</v>
       </c>
       <c r="E30" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G30">
         <v>1</v>
@@ -53445,7 +53442,7 @@
         <v>178</v>
       </c>
       <c r="E31" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G31">
         <v>1</v>
@@ -53462,7 +53459,7 @@
         <v>178</v>
       </c>
       <c r="E32" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G32">
         <v>1</v>
@@ -53479,7 +53476,7 @@
         <v>178</v>
       </c>
       <c r="E33" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G33">
         <v>1</v>
@@ -53496,7 +53493,7 @@
         <v>725</v>
       </c>
       <c r="E34" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G34">
         <v>1</v>
@@ -53513,7 +53510,7 @@
         <v>734</v>
       </c>
       <c r="E35" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
       <c r="G35">
         <v>1</v>
@@ -53530,7 +53527,7 @@
         <v>735</v>
       </c>
       <c r="E36" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="G36">
         <v>1</v>
@@ -53547,7 +53544,7 @@
         <v>736</v>
       </c>
       <c r="E37" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="G37">
         <v>1</v>
@@ -53561,10 +53558,10 @@
         <v>79</v>
       </c>
       <c r="D38" t="s">
+        <v>1475</v>
+      </c>
+      <c r="E38" t="s">
         <v>1476</v>
-      </c>
-      <c r="E38" t="s">
-        <v>1477</v>
       </c>
       <c r="G38">
         <v>1</v>
@@ -53578,10 +53575,10 @@
         <v>79</v>
       </c>
       <c r="D39" t="s">
+        <v>1477</v>
+      </c>
+      <c r="E39" t="s">
         <v>1478</v>
-      </c>
-      <c r="E39" t="s">
-        <v>1479</v>
       </c>
       <c r="G39">
         <v>1</v>
@@ -53595,10 +53592,10 @@
         <v>79</v>
       </c>
       <c r="D40" t="s">
+        <v>1479</v>
+      </c>
+      <c r="E40" t="s">
         <v>1480</v>
-      </c>
-      <c r="E40" t="s">
-        <v>1481</v>
       </c>
       <c r="G40">
         <v>1</v>
@@ -53615,7 +53612,7 @@
         <v>178</v>
       </c>
       <c r="E41" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G41">
         <v>1</v>
@@ -53632,7 +53629,7 @@
         <v>725</v>
       </c>
       <c r="E42" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G42">
         <v>2</v>
@@ -53649,7 +53646,7 @@
         <v>178</v>
       </c>
       <c r="E43" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G43">
         <v>1</v>
@@ -53666,7 +53663,7 @@
         <v>178</v>
       </c>
       <c r="E44" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="G44">
         <v>1</v>
@@ -53683,7 +53680,7 @@
         <v>737</v>
       </c>
       <c r="E45" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
       <c r="G45">
         <v>2</v>
@@ -53700,7 +53697,7 @@
         <v>738</v>
       </c>
       <c r="E46" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
       <c r="G46">
         <v>3</v>
@@ -53717,7 +53714,7 @@
         <v>178</v>
       </c>
       <c r="E47" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="G47">
         <v>1</v>
@@ -53768,7 +53765,7 @@
         <v>178</v>
       </c>
       <c r="E50" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G50">
         <v>1</v>
@@ -53785,7 +53782,7 @@
         <v>725</v>
       </c>
       <c r="E51" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G51">
         <v>1</v>
@@ -53802,7 +53799,7 @@
         <v>178</v>
       </c>
       <c r="E52" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G52">
         <v>1</v>
@@ -53819,7 +53816,7 @@
         <v>178</v>
       </c>
       <c r="E53" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G53">
         <v>1</v>
@@ -53836,7 +53833,7 @@
         <v>725</v>
       </c>
       <c r="E54" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G54">
         <v>2</v>
@@ -53853,7 +53850,7 @@
         <v>725</v>
       </c>
       <c r="E55" t="s">
-        <v>1485</v>
+        <v>1484</v>
       </c>
       <c r="G55">
         <v>1</v>
@@ -53870,7 +53867,7 @@
         <v>178</v>
       </c>
       <c r="E56" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G56">
         <v>1</v>
@@ -53887,7 +53884,7 @@
         <v>178</v>
       </c>
       <c r="E57" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G57">
         <v>1</v>
@@ -53904,7 +53901,7 @@
         <v>725</v>
       </c>
       <c r="E58" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G58">
         <v>1</v>
@@ -53921,7 +53918,7 @@
         <v>178</v>
       </c>
       <c r="E59" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G59">
         <v>1</v>
@@ -53938,7 +53935,7 @@
         <v>742</v>
       </c>
       <c r="E60" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
       <c r="G60">
         <v>1</v>
@@ -53955,7 +53952,7 @@
         <v>178</v>
       </c>
       <c r="E61" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G61">
         <v>1</v>
@@ -54023,7 +54020,7 @@
         <v>178</v>
       </c>
       <c r="E65" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G65">
         <v>1</v>
@@ -54040,7 +54037,7 @@
         <v>178</v>
       </c>
       <c r="E66" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="G66">
         <v>1</v>
@@ -54057,7 +54054,7 @@
         <v>746</v>
       </c>
       <c r="E67" t="s">
-        <v>1487</v>
+        <v>1486</v>
       </c>
       <c r="G67">
         <v>2</v>
@@ -54074,7 +54071,7 @@
         <v>725</v>
       </c>
       <c r="E68" t="s">
-        <v>1485</v>
+        <v>1484</v>
       </c>
       <c r="G68">
         <v>1</v>
@@ -54091,7 +54088,7 @@
         <v>178</v>
       </c>
       <c r="E69" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G69">
         <v>1</v>
@@ -54108,7 +54105,7 @@
         <v>178</v>
       </c>
       <c r="E70" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G70">
         <v>1</v>
@@ -54125,7 +54122,7 @@
         <v>725</v>
       </c>
       <c r="E71" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G71">
         <v>1</v>
@@ -54142,7 +54139,7 @@
         <v>178</v>
       </c>
       <c r="E72" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G72">
         <v>1</v>
@@ -54159,7 +54156,7 @@
         <v>178</v>
       </c>
       <c r="E73" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G73">
         <v>1</v>
@@ -54176,7 +54173,7 @@
         <v>178</v>
       </c>
       <c r="E74" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G74">
         <v>1</v>
@@ -54193,7 +54190,7 @@
         <v>725</v>
       </c>
       <c r="E75" t="s">
-        <v>1485</v>
+        <v>1484</v>
       </c>
       <c r="G75">
         <v>2</v>
@@ -54210,7 +54207,7 @@
         <v>178</v>
       </c>
       <c r="E76" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G76">
         <v>1</v>
@@ -54227,7 +54224,7 @@
         <v>178</v>
       </c>
       <c r="E77" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G77">
         <v>1</v>
@@ -54244,7 +54241,7 @@
         <v>178</v>
       </c>
       <c r="E78" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="G78">
         <v>1</v>
@@ -54261,7 +54258,7 @@
         <v>178</v>
       </c>
       <c r="E79" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G79">
         <v>1</v>
@@ -54278,7 +54275,7 @@
         <v>178</v>
       </c>
       <c r="E80" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="G80">
         <v>1</v>
@@ -54295,7 +54292,7 @@
         <v>178</v>
       </c>
       <c r="E81" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="G81">
         <v>1</v>
@@ -54312,7 +54309,7 @@
         <v>178</v>
       </c>
       <c r="E82" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G82">
         <v>1</v>
@@ -54329,7 +54326,7 @@
         <v>178</v>
       </c>
       <c r="E83" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G83">
         <v>1</v>
@@ -54346,7 +54343,7 @@
         <v>178</v>
       </c>
       <c r="E84" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G84">
         <v>1</v>
@@ -54363,7 +54360,7 @@
         <v>725</v>
       </c>
       <c r="E85" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G85">
         <v>1</v>
@@ -54380,7 +54377,7 @@
         <v>178</v>
       </c>
       <c r="E86" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G86">
         <v>1</v>
@@ -54397,7 +54394,7 @@
         <v>178</v>
       </c>
       <c r="E87" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G87">
         <v>1</v>
@@ -54448,7 +54445,7 @@
         <v>178</v>
       </c>
       <c r="E90" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G90">
         <v>1</v>
@@ -54465,7 +54462,7 @@
         <v>725</v>
       </c>
       <c r="E91" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G91">
         <v>1</v>
@@ -54482,7 +54479,7 @@
         <v>178</v>
       </c>
       <c r="E92" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G92">
         <v>1</v>
@@ -54499,7 +54496,7 @@
         <v>725</v>
       </c>
       <c r="E93" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="G93">
         <v>1</v>
@@ -54516,7 +54513,7 @@
         <v>178</v>
       </c>
       <c r="E94" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G94">
         <v>1</v>
@@ -54533,7 +54530,7 @@
         <v>178</v>
       </c>
       <c r="E95" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G95">
         <v>1</v>
@@ -54551,7 +54548,7 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -54562,25 +54559,25 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
+        <v>1488</v>
+      </c>
+      <c r="D3" t="s">
         <v>1489</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1490</v>
       </c>
       <c r="E3" t="s">
         <v>3</v>
       </c>
       <c r="F3" t="s">
+        <v>1490</v>
+      </c>
+      <c r="G3" t="s">
         <v>1491</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>1492</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>1493</v>
-      </c>
-      <c r="I3" t="s">
-        <v>1494</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -54591,7 +54588,7 @@
         <v>712</v>
       </c>
       <c r="D4" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="E4" t="s">
         <v>114</v>
@@ -54603,7 +54600,7 @@
         <v>405</v>
       </c>
       <c r="H4" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -54611,7 +54608,7 @@
         <v>42736</v>
       </c>
       <c r="C5" t="s">
-        <v>1497</v>
+        <v>1496</v>
       </c>
       <c r="E5" t="s">
         <v>114</v>
@@ -54631,19 +54628,19 @@
         <v>42736</v>
       </c>
       <c r="C6" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
       <c r="E6" t="s">
         <v>114</v>
       </c>
       <c r="F6" t="s">
+        <v>1498</v>
+      </c>
+      <c r="G6" t="s">
         <v>1499</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>1500</v>
-      </c>
-      <c r="H6" t="s">
-        <v>1501</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -54651,13 +54648,13 @@
         <v>42736</v>
       </c>
       <c r="C7" t="s">
-        <v>1502</v>
+        <v>1501</v>
       </c>
       <c r="E7" t="s">
         <v>114</v>
       </c>
       <c r="F7" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
       <c r="G7" t="s">
         <v>517</v>
@@ -54711,7 +54708,7 @@
         <v>42736</v>
       </c>
       <c r="C10" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="E10" t="s">
         <v>114</v>
@@ -54723,7 +54720,7 @@
         <v>404</v>
       </c>
       <c r="H10" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -54731,7 +54728,7 @@
         <v>42736</v>
       </c>
       <c r="C11" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
       <c r="E11" t="s">
         <v>114</v>
@@ -54743,7 +54740,7 @@
         <v>404</v>
       </c>
       <c r="H11" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -54751,7 +54748,7 @@
         <v>42736</v>
       </c>
       <c r="C12" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
       <c r="E12" t="s">
         <v>114</v>
@@ -54763,7 +54760,7 @@
         <v>404</v>
       </c>
       <c r="H12" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -54771,7 +54768,7 @@
         <v>42736</v>
       </c>
       <c r="C13" t="s">
-        <v>1507</v>
+        <v>1506</v>
       </c>
       <c r="E13" t="s">
         <v>114</v>
@@ -54783,7 +54780,7 @@
         <v>404</v>
       </c>
       <c r="H13" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -54791,7 +54788,7 @@
         <v>42736</v>
       </c>
       <c r="C14" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E14" t="s">
         <v>114</v>
@@ -54803,7 +54800,7 @@
         <v>404</v>
       </c>
       <c r="H14" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -54811,7 +54808,7 @@
         <v>42736</v>
       </c>
       <c r="C15" t="s">
-        <v>1509</v>
+        <v>1508</v>
       </c>
       <c r="E15" t="s">
         <v>114</v>
@@ -54823,7 +54820,7 @@
         <v>404</v>
       </c>
       <c r="H15" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -54874,7 +54871,7 @@
         <v>712</v>
       </c>
       <c r="D18" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="E18" t="s">
         <v>55</v>
@@ -54886,10 +54883,10 @@
         <v>405</v>
       </c>
       <c r="H18" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="I18" t="s">
-        <v>1510</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -54900,7 +54897,7 @@
         <v>712</v>
       </c>
       <c r="D19" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="E19" t="s">
         <v>55</v>
@@ -54912,10 +54909,10 @@
         <v>404</v>
       </c>
       <c r="H19" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="I19" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -54923,7 +54920,7 @@
         <v>42736</v>
       </c>
       <c r="C20" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="E20" t="s">
         <v>55</v>
@@ -54935,10 +54932,10 @@
         <v>404</v>
       </c>
       <c r="H20" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="I20" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -54946,7 +54943,7 @@
         <v>42736</v>
       </c>
       <c r="C21" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="E21" t="s">
         <v>111</v>
@@ -54958,7 +54955,7 @@
         <v>404</v>
       </c>
       <c r="H21" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -54978,7 +54975,7 @@
         <v>404</v>
       </c>
       <c r="H22" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -54986,7 +54983,7 @@
         <v>42736</v>
       </c>
       <c r="C23" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="E23" t="s">
         <v>49</v>
@@ -54998,7 +54995,7 @@
         <v>404</v>
       </c>
       <c r="H23" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -55006,7 +55003,7 @@
         <v>42736</v>
       </c>
       <c r="C24" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="E24" t="s">
         <v>49</v>
@@ -55018,10 +55015,10 @@
         <v>404</v>
       </c>
       <c r="H24" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="I24" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -55041,7 +55038,7 @@
         <v>404</v>
       </c>
       <c r="H25" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -55061,10 +55058,10 @@
         <v>404</v>
       </c>
       <c r="H26" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="I26" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -55072,7 +55069,7 @@
         <v>42736</v>
       </c>
       <c r="C27" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E27" t="s">
         <v>104</v>
@@ -55092,7 +55089,7 @@
         <v>42736</v>
       </c>
       <c r="C28" t="s">
-        <v>1512</v>
+        <v>1511</v>
       </c>
       <c r="E28" t="s">
         <v>104</v>
@@ -55112,7 +55109,7 @@
         <v>42736</v>
       </c>
       <c r="C29" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="E29" t="s">
         <v>104</v>
@@ -55132,7 +55129,7 @@
         <v>42736</v>
       </c>
       <c r="C30" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E30" t="s">
         <v>42</v>
@@ -55152,7 +55149,7 @@
         <v>42736</v>
       </c>
       <c r="C31" t="s">
-        <v>1512</v>
+        <v>1511</v>
       </c>
       <c r="E31" t="s">
         <v>42</v>
@@ -55172,7 +55169,7 @@
         <v>42736</v>
       </c>
       <c r="C32" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="E32" t="s">
         <v>42</v>
@@ -55192,7 +55189,7 @@
         <v>42736</v>
       </c>
       <c r="C33" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E33" t="s">
         <v>53</v>
@@ -55212,7 +55209,7 @@
         <v>42736</v>
       </c>
       <c r="C34" t="s">
-        <v>1512</v>
+        <v>1511</v>
       </c>
       <c r="E34" t="s">
         <v>53</v>
@@ -55232,7 +55229,7 @@
         <v>42736</v>
       </c>
       <c r="C35" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E35" t="s">
         <v>159</v>
@@ -55272,7 +55269,7 @@
         <v>42736</v>
       </c>
       <c r="C37" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E37" t="s">
         <v>75</v>
@@ -55332,7 +55329,7 @@
         <v>42736</v>
       </c>
       <c r="C40" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E40" t="s">
         <v>46</v>
@@ -55392,7 +55389,7 @@
         <v>42736</v>
       </c>
       <c r="C43" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
       <c r="E43" t="s">
         <v>46</v>
@@ -55412,7 +55409,7 @@
         <v>42736</v>
       </c>
       <c r="C44" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E44" t="s">
         <v>160</v>
@@ -55432,7 +55429,7 @@
         <v>42736</v>
       </c>
       <c r="C45" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="E45" t="s">
         <v>160</v>
@@ -55492,7 +55489,7 @@
         <v>42736</v>
       </c>
       <c r="C48" t="s">
-        <v>1509</v>
+        <v>1508</v>
       </c>
       <c r="E48" t="s">
         <v>98</v>
@@ -55512,7 +55509,7 @@
         <v>42736</v>
       </c>
       <c r="C49" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="E49" t="s">
         <v>98</v>
@@ -55572,7 +55569,7 @@
         <v>42736</v>
       </c>
       <c r="C52" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E52" t="s">
         <v>98</v>
@@ -55584,7 +55581,7 @@
         <v>404</v>
       </c>
       <c r="H52" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
   </sheetData>
@@ -55599,7 +55596,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>1514</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -56945,6 +56942,7 @@
   <dimension ref="A1:Q315"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
+    <col min="3" max="3" width="21.6640625" customWidth="1"/>
     <col min="4" max="4" width="33.1640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -64383,7 +64381,7 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>1515</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -64397,7 +64395,7 @@
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>1516</v>
+        <v>1515</v>
       </c>
       <c r="E3" t="s">
         <v>4</v>
@@ -64418,7 +64416,7 @@
         <v>8</v>
       </c>
       <c r="K3" t="s">
-        <v>1517</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -64435,16 +64433,16 @@
         <v>47</v>
       </c>
       <c r="G4" t="s">
+        <v>1517</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
         <v>1518</v>
       </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>1519</v>
-      </c>
-      <c r="K4" t="s">
-        <v>1520</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -64461,13 +64459,13 @@
         <v>134</v>
       </c>
       <c r="G5" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="H5">
         <v>2</v>
       </c>
       <c r="K5" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -64484,13 +64482,13 @@
         <v>942</v>
       </c>
       <c r="G6" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
       <c r="H6">
         <v>3</v>
       </c>
       <c r="K6" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -64507,16 +64505,16 @@
         <v>47</v>
       </c>
       <c r="G7" t="s">
+        <v>1517</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
         <v>1518</v>
       </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="K7" t="s">
         <v>1519</v>
-      </c>
-      <c r="K7" t="s">
-        <v>1520</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -64533,16 +64531,16 @@
         <v>47</v>
       </c>
       <c r="G8" t="s">
+        <v>1517</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
         <v>1518</v>
       </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="K8" t="s">
         <v>1519</v>
-      </c>
-      <c r="K8" t="s">
-        <v>1520</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -64559,16 +64557,16 @@
         <v>99</v>
       </c>
       <c r="G9" t="s">
+        <v>1517</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
         <v>1518</v>
       </c>
-      <c r="H9">
-        <v>1</v>
-      </c>
-      <c r="I9" t="s">
+      <c r="K9" t="s">
         <v>1519</v>
-      </c>
-      <c r="K9" t="s">
-        <v>1520</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -64585,13 +64583,13 @@
         <v>942</v>
       </c>
       <c r="G10" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
       <c r="H10">
         <v>2</v>
       </c>
       <c r="K10" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -64608,16 +64606,16 @@
         <v>298</v>
       </c>
       <c r="G11" t="s">
-        <v>1523</v>
+        <v>1522</v>
       </c>
       <c r="H11">
         <v>1</v>
       </c>
       <c r="I11" t="s">
+        <v>1518</v>
+      </c>
+      <c r="K11" t="s">
         <v>1519</v>
-      </c>
-      <c r="K11" t="s">
-        <v>1520</v>
       </c>
     </row>
   </sheetData>
@@ -64632,7 +64630,7 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>1524</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -64649,10 +64647,10 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
+        <v>1524</v>
+      </c>
+      <c r="F3" t="s">
         <v>1525</v>
-      </c>
-      <c r="F3" t="s">
-        <v>1526</v>
       </c>
       <c r="G3" t="s">
         <v>8</v>
@@ -64661,10 +64659,10 @@
         <v>583</v>
       </c>
       <c r="I3" t="s">
+        <v>1526</v>
+      </c>
+      <c r="J3" t="s">
         <v>1527</v>
-      </c>
-      <c r="J3" t="s">
-        <v>1528</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -64672,13 +64670,13 @@
         <v>103</v>
       </c>
       <c r="C4" t="s">
+        <v>1528</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
         <v>1529</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>1530</v>
       </c>
       <c r="F4" t="s">
         <v>199</v>
@@ -64687,13 +64685,13 @@
         <v>1289</v>
       </c>
       <c r="H4" t="s">
+        <v>1530</v>
+      </c>
+      <c r="I4" t="s">
         <v>1531</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>1532</v>
-      </c>
-      <c r="J4" t="s">
-        <v>1533</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -64701,13 +64699,13 @@
         <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="D5">
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>1534</v>
+        <v>1533</v>
       </c>
       <c r="F5" t="s">
         <v>202</v>
@@ -64716,10 +64714,10 @@
         <v>1289</v>
       </c>
       <c r="H5" t="s">
+        <v>1534</v>
+      </c>
+      <c r="I5" t="s">
         <v>1535</v>
-      </c>
-      <c r="I5" t="s">
-        <v>1536</v>
       </c>
       <c r="J5" t="s">
         <v>514</v>
@@ -64730,13 +64728,13 @@
         <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="D6">
         <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>1537</v>
+        <v>1536</v>
       </c>
       <c r="F6" t="s">
         <v>202</v>
@@ -64745,10 +64743,10 @@
         <v>1289</v>
       </c>
       <c r="H6" t="s">
+        <v>1537</v>
+      </c>
+      <c r="I6" t="s">
         <v>1538</v>
-      </c>
-      <c r="I6" t="s">
-        <v>1539</v>
       </c>
       <c r="J6" t="s">
         <v>517</v>
@@ -64759,25 +64757,25 @@
         <v>103</v>
       </c>
       <c r="C7" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="D7">
         <v>4</v>
       </c>
       <c r="E7" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F7" t="s">
         <v>1541</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
+        <v>1537</v>
+      </c>
+      <c r="I7" t="s">
         <v>1542</v>
       </c>
-      <c r="H7" t="s">
-        <v>1538</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>1543</v>
-      </c>
-      <c r="J7" t="s">
-        <v>1544</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -64785,25 +64783,25 @@
         <v>110</v>
       </c>
       <c r="C8" t="s">
-        <v>1545</v>
+        <v>1544</v>
       </c>
       <c r="D8">
         <v>5</v>
       </c>
       <c r="E8" t="s">
-        <v>1541</v>
+        <v>1540</v>
       </c>
       <c r="F8" t="s">
         <v>224</v>
       </c>
       <c r="H8" t="s">
+        <v>1545</v>
+      </c>
+      <c r="I8" t="s">
         <v>1546</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>1547</v>
-      </c>
-      <c r="J8" t="s">
-        <v>1548</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -64811,25 +64809,25 @@
         <v>150</v>
       </c>
       <c r="C9" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="D9">
         <v>6</v>
       </c>
       <c r="E9" t="s">
-        <v>1530</v>
+        <v>1529</v>
       </c>
       <c r="F9" t="s">
         <v>224</v>
       </c>
       <c r="H9" t="s">
+        <v>1548</v>
+      </c>
+      <c r="I9" t="s">
         <v>1549</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>1550</v>
-      </c>
-      <c r="J9" t="s">
-        <v>1551</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -64837,13 +64835,13 @@
         <v>150</v>
       </c>
       <c r="C10" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="D10">
         <v>7</v>
       </c>
       <c r="E10" t="s">
-        <v>1552</v>
+        <v>1551</v>
       </c>
       <c r="F10" t="s">
         <v>199</v>
@@ -64852,10 +64850,10 @@
         <v>1289</v>
       </c>
       <c r="H10" t="s">
+        <v>1552</v>
+      </c>
+      <c r="I10" t="s">
         <v>1553</v>
-      </c>
-      <c r="I10" t="s">
-        <v>1554</v>
       </c>
       <c r="J10" t="s">
         <v>517</v>
@@ -64866,25 +64864,25 @@
         <v>151</v>
       </c>
       <c r="C11" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="D11">
         <v>8</v>
       </c>
       <c r="E11" t="s">
-        <v>1530</v>
+        <v>1529</v>
       </c>
       <c r="F11" t="s">
         <v>224</v>
       </c>
       <c r="H11" t="s">
-        <v>1549</v>
+        <v>1548</v>
       </c>
       <c r="I11" t="s">
+        <v>1554</v>
+      </c>
+      <c r="J11" t="s">
         <v>1555</v>
-      </c>
-      <c r="J11" t="s">
-        <v>1556</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -64892,22 +64890,22 @@
         <v>140</v>
       </c>
       <c r="C12" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="D12">
         <v>9</v>
       </c>
       <c r="E12" t="s">
-        <v>1530</v>
+        <v>1529</v>
       </c>
       <c r="F12" t="s">
         <v>224</v>
       </c>
       <c r="H12" t="s">
-        <v>1549</v>
+        <v>1548</v>
       </c>
       <c r="I12" t="s">
-        <v>1557</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -64915,13 +64913,13 @@
         <v>98</v>
       </c>
       <c r="C13" t="s">
+        <v>1528</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
         <v>1529</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
-        <v>1530</v>
       </c>
       <c r="F13" t="s">
         <v>199</v>
@@ -64930,13 +64928,13 @@
         <v>1289</v>
       </c>
       <c r="H13" t="s">
+        <v>1530</v>
+      </c>
+      <c r="I13" t="s">
         <v>1531</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>1532</v>
-      </c>
-      <c r="J13" t="s">
-        <v>1533</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -64944,13 +64942,13 @@
         <v>98</v>
       </c>
       <c r="C14" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="D14">
         <v>2</v>
       </c>
       <c r="E14" t="s">
-        <v>1534</v>
+        <v>1533</v>
       </c>
       <c r="F14" t="s">
         <v>202</v>
@@ -64959,10 +64957,10 @@
         <v>1289</v>
       </c>
       <c r="H14" t="s">
+        <v>1534</v>
+      </c>
+      <c r="I14" t="s">
         <v>1535</v>
-      </c>
-      <c r="I14" t="s">
-        <v>1536</v>
       </c>
       <c r="J14" t="s">
         <v>514</v>
@@ -64973,13 +64971,13 @@
         <v>98</v>
       </c>
       <c r="C15" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="D15">
         <v>3</v>
       </c>
       <c r="E15" t="s">
-        <v>1537</v>
+        <v>1536</v>
       </c>
       <c r="F15" t="s">
         <v>202</v>
@@ -64988,10 +64986,10 @@
         <v>1289</v>
       </c>
       <c r="H15" t="s">
+        <v>1537</v>
+      </c>
+      <c r="I15" t="s">
         <v>1538</v>
-      </c>
-      <c r="I15" t="s">
-        <v>1539</v>
       </c>
       <c r="J15" t="s">
         <v>517</v>
@@ -67427,7 +67425,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="113" spans="1:13">
+    <row r="113" spans="1:16">
       <c r="A113" s="1">
         <v>42741</v>
       </c>
@@ -67447,7 +67445,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="114" spans="1:13">
+    <row r="114" spans="1:16">
       <c r="A114" s="1">
         <v>42742</v>
       </c>
@@ -67470,7 +67468,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="115" spans="1:13">
+    <row r="115" spans="1:16">
       <c r="A115" s="1">
         <v>42742</v>
       </c>
@@ -67490,7 +67488,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="116" spans="1:13">
+    <row r="116" spans="1:16">
       <c r="A116" s="1">
         <v>42742</v>
       </c>
@@ -67510,7 +67508,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="117" spans="1:13">
+    <row r="117" spans="1:16">
       <c r="A117" s="1">
         <v>42736</v>
       </c>
@@ -67528,6 +67526,9 @@
       </c>
       <c r="M117" t="s">
         <v>218</v>
+      </c>
+      <c r="P117" t="s">
+        <v>1557</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CCD-8328: Updated with master
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16262" uniqueCount="1563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16269" uniqueCount="1563">
   <si>
     <t>SearchInputFields</t>
   </si>
@@ -26443,7 +26443,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O284"/>
+  <dimension ref="A1:P285"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -26498,6 +26498,9 @@
       <c r="O3" t="s">
         <v>1224</v>
       </c>
+      <c r="P3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n" s="22">
@@ -26529,6 +26532,7 @@
       <c r="M4"/>
       <c r="N4"/>
       <c r="O4"/>
+      <c r="P4"/>
     </row>
     <row r="5">
       <c r="A5" t="n" s="22">
@@ -26560,6 +26564,7 @@
       <c r="M5"/>
       <c r="N5"/>
       <c r="O5"/>
+      <c r="P5"/>
     </row>
     <row r="6">
       <c r="A6" t="n" s="22">
@@ -26591,6 +26596,7 @@
       <c r="M6"/>
       <c r="N6"/>
       <c r="O6"/>
+      <c r="P6"/>
     </row>
     <row r="7">
       <c r="A7" t="n" s="22">
@@ -26622,6 +26628,7 @@
       <c r="M7"/>
       <c r="N7"/>
       <c r="O7"/>
+      <c r="P7"/>
     </row>
     <row r="8">
       <c r="A8" t="n" s="22">
@@ -26653,6 +26660,7 @@
       <c r="M8"/>
       <c r="N8"/>
       <c r="O8"/>
+      <c r="P8"/>
     </row>
     <row r="9">
       <c r="A9" t="n" s="22">
@@ -26684,6 +26692,7 @@
       <c r="M9"/>
       <c r="N9"/>
       <c r="O9"/>
+      <c r="P9"/>
     </row>
     <row r="10">
       <c r="A10" t="n" s="22">
@@ -26715,6 +26724,7 @@
       <c r="M10"/>
       <c r="N10"/>
       <c r="O10"/>
+      <c r="P10"/>
     </row>
     <row r="11">
       <c r="A11" t="n" s="22">
@@ -26746,6 +26756,7 @@
       <c r="M11"/>
       <c r="N11"/>
       <c r="O11"/>
+      <c r="P11"/>
     </row>
     <row r="12">
       <c r="A12" t="n" s="22">
@@ -26777,6 +26788,7 @@
       <c r="M12"/>
       <c r="N12"/>
       <c r="O12"/>
+      <c r="P12"/>
     </row>
     <row r="13">
       <c r="A13" t="n" s="22">
@@ -26808,6 +26820,7 @@
       <c r="M13"/>
       <c r="N13"/>
       <c r="O13"/>
+      <c r="P13"/>
     </row>
     <row r="14">
       <c r="A14" t="n" s="22">
@@ -26841,6 +26854,7 @@
       <c r="M14"/>
       <c r="N14"/>
       <c r="O14"/>
+      <c r="P14"/>
     </row>
     <row r="15">
       <c r="A15" t="n" s="22">
@@ -26876,6 +26890,7 @@
       <c r="M15"/>
       <c r="N15"/>
       <c r="O15"/>
+      <c r="P15"/>
     </row>
     <row r="16">
       <c r="A16" t="n" s="22">
@@ -26907,6 +26922,7 @@
       <c r="M16"/>
       <c r="N16"/>
       <c r="O16"/>
+      <c r="P16"/>
     </row>
     <row r="17">
       <c r="A17" t="n" s="22">
@@ -26938,6 +26954,7 @@
       <c r="M17"/>
       <c r="N17"/>
       <c r="O17"/>
+      <c r="P17"/>
     </row>
     <row r="18">
       <c r="A18" t="n" s="22">
@@ -26969,6 +26986,7 @@
       <c r="M18"/>
       <c r="N18"/>
       <c r="O18"/>
+      <c r="P18"/>
     </row>
     <row r="19">
       <c r="A19" t="n" s="22">
@@ -27002,6 +27020,7 @@
       <c r="M19"/>
       <c r="N19"/>
       <c r="O19"/>
+      <c r="P19"/>
     </row>
     <row r="20">
       <c r="A20" t="n" s="22">
@@ -27033,6 +27052,7 @@
       <c r="M20"/>
       <c r="N20"/>
       <c r="O20"/>
+      <c r="P20"/>
     </row>
     <row r="21">
       <c r="A21" t="n" s="22">
@@ -27070,6 +27090,7 @@
       <c r="O21" t="s">
         <v>1241</v>
       </c>
+      <c r="P21"/>
     </row>
     <row r="22">
       <c r="A22" t="n" s="22">
@@ -27103,6 +27124,7 @@
       <c r="M22"/>
       <c r="N22"/>
       <c r="O22"/>
+      <c r="P22"/>
     </row>
     <row r="23">
       <c r="A23" t="n" s="22">
@@ -27134,6 +27156,7 @@
       <c r="M23"/>
       <c r="N23"/>
       <c r="O23"/>
+      <c r="P23"/>
     </row>
     <row r="24">
       <c r="A24" t="n" s="22">
@@ -27165,6 +27188,7 @@
       <c r="M24"/>
       <c r="N24"/>
       <c r="O24"/>
+      <c r="P24"/>
     </row>
     <row r="25">
       <c r="A25" t="n" s="22">
@@ -27198,6 +27222,7 @@
       <c r="M25"/>
       <c r="N25"/>
       <c r="O25"/>
+      <c r="P25"/>
     </row>
     <row r="26">
       <c r="A26" t="n" s="22">
@@ -27229,6 +27254,7 @@
       <c r="M26"/>
       <c r="N26"/>
       <c r="O26"/>
+      <c r="P26"/>
     </row>
     <row r="27">
       <c r="A27" t="n" s="22">
@@ -27260,6 +27286,7 @@
       <c r="M27"/>
       <c r="N27"/>
       <c r="O27"/>
+      <c r="P27"/>
     </row>
     <row r="28">
       <c r="A28" t="n" s="22">
@@ -27291,6 +27318,7 @@
       <c r="M28"/>
       <c r="N28"/>
       <c r="O28"/>
+      <c r="P28"/>
     </row>
     <row r="29">
       <c r="A29" t="n" s="22">
@@ -27322,6 +27350,7 @@
       <c r="M29"/>
       <c r="N29"/>
       <c r="O29"/>
+      <c r="P29"/>
     </row>
     <row r="30">
       <c r="A30" t="n" s="22">
@@ -27353,6 +27382,7 @@
       <c r="M30"/>
       <c r="N30"/>
       <c r="O30"/>
+      <c r="P30"/>
     </row>
     <row r="31">
       <c r="A31" t="n" s="22">
@@ -27384,6 +27414,7 @@
       <c r="M31"/>
       <c r="N31"/>
       <c r="O31"/>
+      <c r="P31"/>
     </row>
     <row r="32">
       <c r="A32" t="n" s="22">
@@ -27415,6 +27446,7 @@
       <c r="M32"/>
       <c r="N32"/>
       <c r="O32"/>
+      <c r="P32"/>
     </row>
     <row r="33">
       <c r="A33" t="n" s="22">
@@ -27446,6 +27478,7 @@
       <c r="M33"/>
       <c r="N33"/>
       <c r="O33"/>
+      <c r="P33"/>
     </row>
     <row r="34">
       <c r="A34" t="n" s="22">
@@ -27477,6 +27510,7 @@
       <c r="M34"/>
       <c r="N34"/>
       <c r="O34"/>
+      <c r="P34"/>
     </row>
     <row r="35">
       <c r="A35" t="n" s="22">
@@ -27508,6 +27542,7 @@
       <c r="M35"/>
       <c r="N35"/>
       <c r="O35"/>
+      <c r="P35"/>
     </row>
     <row r="36">
       <c r="A36" t="n" s="22">
@@ -27539,6 +27574,7 @@
       <c r="M36"/>
       <c r="N36"/>
       <c r="O36"/>
+      <c r="P36"/>
     </row>
     <row r="37">
       <c r="A37" t="n" s="22">
@@ -27574,6 +27610,7 @@
       <c r="O37" t="s">
         <v>1241</v>
       </c>
+      <c r="P37"/>
     </row>
     <row r="38">
       <c r="A38" t="n" s="22">
@@ -27605,6 +27642,7 @@
       <c r="M38"/>
       <c r="N38"/>
       <c r="O38"/>
+      <c r="P38"/>
     </row>
     <row r="39">
       <c r="A39" t="n" s="22">
@@ -27636,6 +27674,7 @@
       <c r="M39"/>
       <c r="N39"/>
       <c r="O39"/>
+      <c r="P39"/>
     </row>
     <row r="40">
       <c r="A40" t="n" s="22">
@@ -27667,6 +27706,7 @@
       <c r="M40"/>
       <c r="N40"/>
       <c r="O40"/>
+      <c r="P40"/>
     </row>
     <row r="41">
       <c r="A41" t="n" s="22">
@@ -27700,6 +27740,7 @@
       <c r="M41"/>
       <c r="N41"/>
       <c r="O41"/>
+      <c r="P41"/>
     </row>
     <row r="42">
       <c r="A42" t="n" s="22">
@@ -27731,6 +27772,7 @@
       <c r="M42"/>
       <c r="N42"/>
       <c r="O42"/>
+      <c r="P42"/>
     </row>
     <row r="43">
       <c r="A43" t="n" s="22">
@@ -27762,6 +27804,7 @@
       <c r="M43"/>
       <c r="N43"/>
       <c r="O43"/>
+      <c r="P43"/>
     </row>
     <row r="44">
       <c r="A44" t="n" s="22">
@@ -27793,6 +27836,7 @@
       <c r="M44"/>
       <c r="N44"/>
       <c r="O44"/>
+      <c r="P44"/>
     </row>
     <row r="45">
       <c r="A45" t="n" s="22">
@@ -27824,6 +27868,7 @@
       <c r="M45"/>
       <c r="N45"/>
       <c r="O45"/>
+      <c r="P45"/>
     </row>
     <row r="46">
       <c r="A46" t="n" s="22">
@@ -27855,6 +27900,7 @@
       <c r="M46"/>
       <c r="N46"/>
       <c r="O46"/>
+      <c r="P46"/>
     </row>
     <row r="47">
       <c r="A47" t="n" s="22">
@@ -27886,6 +27932,7 @@
       <c r="M47"/>
       <c r="N47"/>
       <c r="O47"/>
+      <c r="P47"/>
     </row>
     <row r="48">
       <c r="A48" t="n" s="22">
@@ -27917,6 +27964,7 @@
       <c r="M48"/>
       <c r="N48"/>
       <c r="O48"/>
+      <c r="P48"/>
     </row>
     <row r="49">
       <c r="A49" t="n" s="22">
@@ -27948,6 +27996,7 @@
       <c r="M49"/>
       <c r="N49"/>
       <c r="O49"/>
+      <c r="P49"/>
     </row>
     <row r="50">
       <c r="A50" t="n" s="22">
@@ -27979,6 +28028,7 @@
       <c r="M50"/>
       <c r="N50"/>
       <c r="O50"/>
+      <c r="P50"/>
     </row>
     <row r="51">
       <c r="A51" t="n" s="22">
@@ -28010,6 +28060,7 @@
       <c r="M51"/>
       <c r="N51"/>
       <c r="O51"/>
+      <c r="P51"/>
     </row>
     <row r="52">
       <c r="A52" t="n" s="22">
@@ -28041,6 +28092,7 @@
       <c r="M52"/>
       <c r="N52"/>
       <c r="O52"/>
+      <c r="P52"/>
     </row>
     <row r="53">
       <c r="A53" t="n" s="22">
@@ -28072,6 +28124,7 @@
       <c r="M53"/>
       <c r="N53"/>
       <c r="O53"/>
+      <c r="P53"/>
     </row>
     <row r="54">
       <c r="A54" t="n" s="22">
@@ -28103,6 +28156,7 @@
       <c r="M54"/>
       <c r="N54"/>
       <c r="O54"/>
+      <c r="P54"/>
     </row>
     <row r="55">
       <c r="A55" t="n" s="22">
@@ -28136,6 +28190,7 @@
       <c r="M55"/>
       <c r="N55"/>
       <c r="O55"/>
+      <c r="P55"/>
     </row>
     <row r="56">
       <c r="A56" t="n" s="22">
@@ -28167,6 +28222,7 @@
       <c r="M56"/>
       <c r="N56"/>
       <c r="O56"/>
+      <c r="P56"/>
     </row>
     <row r="57">
       <c r="A57" t="n" s="22">
@@ -28198,6 +28254,7 @@
       <c r="M57"/>
       <c r="N57"/>
       <c r="O57"/>
+      <c r="P57"/>
     </row>
     <row r="58">
       <c r="A58" t="n" s="22">
@@ -28229,6 +28286,7 @@
       <c r="M58"/>
       <c r="N58"/>
       <c r="O58"/>
+      <c r="P58"/>
     </row>
     <row r="59">
       <c r="A59" t="n" s="22">
@@ -28262,6 +28320,7 @@
       <c r="M59"/>
       <c r="N59"/>
       <c r="O59"/>
+      <c r="P59"/>
     </row>
     <row r="60">
       <c r="A60" t="n" s="22">
@@ -28293,6 +28352,7 @@
       <c r="M60"/>
       <c r="N60"/>
       <c r="O60"/>
+      <c r="P60"/>
     </row>
     <row r="61">
       <c r="A61" t="n" s="22">
@@ -28324,6 +28384,7 @@
       <c r="M61"/>
       <c r="N61"/>
       <c r="O61"/>
+      <c r="P61"/>
     </row>
     <row r="62">
       <c r="A62" t="n" s="22">
@@ -28355,6 +28416,7 @@
       <c r="M62"/>
       <c r="N62"/>
       <c r="O62"/>
+      <c r="P62"/>
     </row>
     <row r="63">
       <c r="A63" t="n" s="22">
@@ -28388,6 +28450,7 @@
       <c r="M63"/>
       <c r="N63"/>
       <c r="O63"/>
+      <c r="P63"/>
     </row>
     <row r="64">
       <c r="A64" t="n" s="22">
@@ -28419,6 +28482,7 @@
       <c r="M64"/>
       <c r="N64"/>
       <c r="O64"/>
+      <c r="P64"/>
     </row>
     <row r="65">
       <c r="A65" t="n" s="22">
@@ -28450,6 +28514,7 @@
       <c r="M65"/>
       <c r="N65"/>
       <c r="O65"/>
+      <c r="P65"/>
     </row>
     <row r="66">
       <c r="A66" t="n" s="22">
@@ -28481,6 +28546,7 @@
       <c r="M66"/>
       <c r="N66"/>
       <c r="O66"/>
+      <c r="P66"/>
     </row>
     <row r="67">
       <c r="A67" t="n" s="22">
@@ -28514,6 +28580,7 @@
       <c r="M67"/>
       <c r="N67"/>
       <c r="O67"/>
+      <c r="P67"/>
     </row>
     <row r="68">
       <c r="A68" t="n" s="22">
@@ -28545,6 +28612,7 @@
       <c r="M68"/>
       <c r="N68"/>
       <c r="O68"/>
+      <c r="P68"/>
     </row>
     <row r="69">
       <c r="A69" t="n" s="22">
@@ -28578,6 +28646,7 @@
       <c r="M69"/>
       <c r="N69"/>
       <c r="O69"/>
+      <c r="P69"/>
     </row>
     <row r="70">
       <c r="A70" t="n" s="22">
@@ -28611,6 +28680,7 @@
       <c r="M70"/>
       <c r="N70"/>
       <c r="O70"/>
+      <c r="P70"/>
     </row>
     <row r="71">
       <c r="A71" t="n" s="22">
@@ -28642,6 +28712,7 @@
       <c r="M71"/>
       <c r="N71"/>
       <c r="O71"/>
+      <c r="P71"/>
     </row>
     <row r="72">
       <c r="A72" t="n" s="22">
@@ -28673,6 +28744,7 @@
       <c r="M72"/>
       <c r="N72"/>
       <c r="O72"/>
+      <c r="P72"/>
     </row>
     <row r="73">
       <c r="A73" t="n" s="22">
@@ -28704,6 +28776,7 @@
       <c r="M73"/>
       <c r="N73"/>
       <c r="O73"/>
+      <c r="P73"/>
     </row>
     <row r="74">
       <c r="A74" t="n" s="22">
@@ -28735,6 +28808,7 @@
       <c r="M74"/>
       <c r="N74"/>
       <c r="O74"/>
+      <c r="P74"/>
     </row>
     <row r="75">
       <c r="A75" t="n" s="22">
@@ -28766,6 +28840,7 @@
       <c r="M75"/>
       <c r="N75"/>
       <c r="O75"/>
+      <c r="P75"/>
     </row>
     <row r="76">
       <c r="A76" t="n" s="22">
@@ -28797,6 +28872,7 @@
       <c r="M76"/>
       <c r="N76"/>
       <c r="O76"/>
+      <c r="P76"/>
     </row>
     <row r="77">
       <c r="A77" t="n" s="22">
@@ -28828,6 +28904,7 @@
       <c r="M77"/>
       <c r="N77"/>
       <c r="O77"/>
+      <c r="P77"/>
     </row>
     <row r="78">
       <c r="A78" t="n" s="22">
@@ -28859,6 +28936,7 @@
       <c r="M78"/>
       <c r="N78"/>
       <c r="O78"/>
+      <c r="P78"/>
     </row>
     <row r="79">
       <c r="A79" t="n" s="22">
@@ -28890,6 +28968,7 @@
       <c r="M79"/>
       <c r="N79"/>
       <c r="O79"/>
+      <c r="P79"/>
     </row>
     <row r="80">
       <c r="A80" t="n" s="22">
@@ -28921,6 +29000,7 @@
       <c r="M80"/>
       <c r="N80"/>
       <c r="O80"/>
+      <c r="P80"/>
     </row>
     <row r="81">
       <c r="A81" t="n" s="22">
@@ -28952,6 +29032,7 @@
       <c r="M81"/>
       <c r="N81"/>
       <c r="O81"/>
+      <c r="P81"/>
     </row>
     <row r="82">
       <c r="A82" t="n" s="22">
@@ -28983,6 +29064,7 @@
       <c r="M82"/>
       <c r="N82"/>
       <c r="O82"/>
+      <c r="P82"/>
     </row>
     <row r="83">
       <c r="A83" t="n" s="22">
@@ -29014,6 +29096,7 @@
       <c r="M83"/>
       <c r="N83"/>
       <c r="O83"/>
+      <c r="P83"/>
     </row>
     <row r="84">
       <c r="A84" t="n" s="22">
@@ -29045,6 +29128,7 @@
       <c r="M84"/>
       <c r="N84"/>
       <c r="O84"/>
+      <c r="P84"/>
     </row>
     <row r="85">
       <c r="A85" t="n" s="22">
@@ -29074,6 +29158,7 @@
       <c r="M85"/>
       <c r="N85"/>
       <c r="O85"/>
+      <c r="P85"/>
     </row>
     <row r="86">
       <c r="A86" t="n" s="22">
@@ -29103,6 +29188,7 @@
       <c r="M86"/>
       <c r="N86"/>
       <c r="O86"/>
+      <c r="P86"/>
     </row>
     <row r="87">
       <c r="A87" t="n" s="22">
@@ -29132,6 +29218,7 @@
       <c r="M87"/>
       <c r="N87"/>
       <c r="O87"/>
+      <c r="P87"/>
     </row>
     <row r="88">
       <c r="A88" t="n" s="22">
@@ -29161,6 +29248,7 @@
       <c r="M88"/>
       <c r="N88"/>
       <c r="O88"/>
+      <c r="P88"/>
     </row>
     <row r="89">
       <c r="A89" t="n" s="22">
@@ -29190,6 +29278,7 @@
       <c r="M89"/>
       <c r="N89"/>
       <c r="O89"/>
+      <c r="P89"/>
     </row>
     <row r="90">
       <c r="A90" t="n" s="22">
@@ -29219,6 +29308,7 @@
       <c r="M90"/>
       <c r="N90"/>
       <c r="O90"/>
+      <c r="P90"/>
     </row>
     <row r="91">
       <c r="A91" t="n" s="22">
@@ -29250,6 +29340,7 @@
       <c r="M91"/>
       <c r="N91"/>
       <c r="O91"/>
+      <c r="P91"/>
     </row>
     <row r="92">
       <c r="A92" t="n" s="22">
@@ -29279,6 +29370,7 @@
       <c r="M92"/>
       <c r="N92"/>
       <c r="O92"/>
+      <c r="P92"/>
     </row>
     <row r="93">
       <c r="A93" t="n" s="22">
@@ -29310,6 +29402,7 @@
       <c r="M93"/>
       <c r="N93"/>
       <c r="O93"/>
+      <c r="P93"/>
     </row>
     <row r="94">
       <c r="A94" t="n" s="22">
@@ -29339,6 +29432,7 @@
       <c r="M94"/>
       <c r="N94"/>
       <c r="O94"/>
+      <c r="P94"/>
     </row>
     <row r="95">
       <c r="A95" t="n" s="22">
@@ -29370,6 +29464,7 @@
       <c r="M95"/>
       <c r="N95"/>
       <c r="O95"/>
+      <c r="P95"/>
     </row>
     <row r="96">
       <c r="A96" t="n" s="22">
@@ -29399,6 +29494,7 @@
       <c r="M96"/>
       <c r="N96"/>
       <c r="O96"/>
+      <c r="P96"/>
     </row>
     <row r="97">
       <c r="A97" t="n" s="22">
@@ -29428,6 +29524,7 @@
       <c r="M97"/>
       <c r="N97"/>
       <c r="O97"/>
+      <c r="P97"/>
     </row>
     <row r="98">
       <c r="A98" t="n" s="22">
@@ -29459,6 +29556,7 @@
       <c r="M98"/>
       <c r="N98"/>
       <c r="O98"/>
+      <c r="P98"/>
     </row>
     <row r="99">
       <c r="A99" t="n" s="22">
@@ -29488,6 +29586,7 @@
       <c r="M99"/>
       <c r="N99"/>
       <c r="O99"/>
+      <c r="P99"/>
     </row>
     <row r="100">
       <c r="A100" t="n" s="22">
@@ -29517,6 +29616,7 @@
       <c r="M100"/>
       <c r="N100"/>
       <c r="O100"/>
+      <c r="P100"/>
     </row>
     <row r="101">
       <c r="A101" t="n" s="22">
@@ -29548,6 +29648,7 @@
       <c r="M101"/>
       <c r="N101"/>
       <c r="O101"/>
+      <c r="P101"/>
     </row>
     <row r="102">
       <c r="A102" t="n" s="22">
@@ -29579,6 +29680,7 @@
       <c r="M102"/>
       <c r="N102"/>
       <c r="O102"/>
+      <c r="P102"/>
     </row>
     <row r="103">
       <c r="A103" t="n" s="22">
@@ -29610,6 +29712,7 @@
       <c r="M103"/>
       <c r="N103"/>
       <c r="O103"/>
+      <c r="P103"/>
     </row>
     <row r="104">
       <c r="A104" t="n" s="22">
@@ -29641,6 +29744,7 @@
       <c r="M104"/>
       <c r="N104"/>
       <c r="O104"/>
+      <c r="P104"/>
     </row>
     <row r="105">
       <c r="A105" t="n" s="22">
@@ -29672,6 +29776,7 @@
       <c r="M105"/>
       <c r="N105"/>
       <c r="O105"/>
+      <c r="P105"/>
     </row>
     <row r="106">
       <c r="A106" t="n" s="22">
@@ -29703,6 +29808,7 @@
       <c r="M106"/>
       <c r="N106"/>
       <c r="O106"/>
+      <c r="P106"/>
     </row>
     <row r="107">
       <c r="A107" t="n" s="22">
@@ -29734,6 +29840,7 @@
       <c r="M107"/>
       <c r="N107"/>
       <c r="O107"/>
+      <c r="P107"/>
     </row>
     <row r="108">
       <c r="A108" t="n" s="22">
@@ -29767,6 +29874,7 @@
       <c r="M108"/>
       <c r="N108"/>
       <c r="O108"/>
+      <c r="P108"/>
     </row>
     <row r="109">
       <c r="A109" t="n" s="22">
@@ -29800,6 +29908,7 @@
       <c r="M109"/>
       <c r="N109"/>
       <c r="O109"/>
+      <c r="P109"/>
     </row>
     <row r="110">
       <c r="A110" t="n" s="22">
@@ -29831,6 +29940,7 @@
       <c r="M110"/>
       <c r="N110"/>
       <c r="O110"/>
+      <c r="P110"/>
     </row>
     <row r="111">
       <c r="A111" t="n" s="22">
@@ -29862,6 +29972,7 @@
       <c r="M111"/>
       <c r="N111"/>
       <c r="O111"/>
+      <c r="P111"/>
     </row>
     <row r="112">
       <c r="A112" t="n" s="22">
@@ -29893,6 +30004,7 @@
       <c r="M112"/>
       <c r="N112"/>
       <c r="O112"/>
+      <c r="P112"/>
     </row>
     <row r="113">
       <c r="A113" t="n" s="22">
@@ -29926,6 +30038,7 @@
       <c r="M113"/>
       <c r="N113"/>
       <c r="O113"/>
+      <c r="P113"/>
     </row>
     <row r="114">
       <c r="A114" t="n" s="22">
@@ -29959,6 +30072,7 @@
       <c r="M114"/>
       <c r="N114"/>
       <c r="O114"/>
+      <c r="P114"/>
     </row>
     <row r="115">
       <c r="A115" t="n" s="22">
@@ -29990,6 +30104,7 @@
       <c r="M115"/>
       <c r="N115"/>
       <c r="O115"/>
+      <c r="P115"/>
     </row>
     <row r="116">
       <c r="A116" t="n" s="22">
@@ -30021,6 +30136,7 @@
       <c r="M116"/>
       <c r="N116"/>
       <c r="O116"/>
+      <c r="P116"/>
     </row>
     <row r="117">
       <c r="A117" t="n" s="22">
@@ -30052,6 +30168,7 @@
       <c r="M117"/>
       <c r="N117"/>
       <c r="O117"/>
+      <c r="P117"/>
     </row>
     <row r="118">
       <c r="A118" t="n" s="22">
@@ -30085,6 +30202,7 @@
       <c r="M118"/>
       <c r="N118"/>
       <c r="O118"/>
+      <c r="P118"/>
     </row>
     <row r="119">
       <c r="A119" t="n" s="22">
@@ -30118,6 +30236,7 @@
       <c r="M119"/>
       <c r="N119"/>
       <c r="O119"/>
+      <c r="P119"/>
     </row>
     <row r="120">
       <c r="A120" t="n" s="22">
@@ -30149,6 +30268,7 @@
       <c r="M120"/>
       <c r="N120"/>
       <c r="O120"/>
+      <c r="P120"/>
     </row>
     <row r="121">
       <c r="A121" t="n" s="22">
@@ -30180,6 +30300,7 @@
       <c r="M121"/>
       <c r="N121"/>
       <c r="O121"/>
+      <c r="P121"/>
     </row>
     <row r="122">
       <c r="A122" t="n" s="22">
@@ -30211,6 +30332,7 @@
       <c r="M122"/>
       <c r="N122"/>
       <c r="O122"/>
+      <c r="P122"/>
     </row>
     <row r="123">
       <c r="A123" t="n" s="22">
@@ -30244,6 +30366,7 @@
       <c r="M123"/>
       <c r="N123"/>
       <c r="O123"/>
+      <c r="P123"/>
     </row>
     <row r="124">
       <c r="A124" t="n" s="22">
@@ -30277,6 +30400,7 @@
       <c r="M124"/>
       <c r="N124"/>
       <c r="O124"/>
+      <c r="P124"/>
     </row>
     <row r="125">
       <c r="A125" t="n" s="22">
@@ -30308,6 +30432,7 @@
       <c r="M125"/>
       <c r="N125"/>
       <c r="O125"/>
+      <c r="P125"/>
     </row>
     <row r="126">
       <c r="A126" t="n" s="22">
@@ -30339,6 +30464,7 @@
       <c r="M126"/>
       <c r="N126"/>
       <c r="O126"/>
+      <c r="P126"/>
     </row>
     <row r="127">
       <c r="A127" t="n" s="22">
@@ -30370,6 +30496,7 @@
       <c r="M127"/>
       <c r="N127"/>
       <c r="O127"/>
+      <c r="P127"/>
     </row>
     <row r="128">
       <c r="A128" t="n" s="22">
@@ -30403,6 +30530,7 @@
       <c r="M128"/>
       <c r="N128"/>
       <c r="O128"/>
+      <c r="P128"/>
     </row>
     <row r="129">
       <c r="A129" t="n" s="22">
@@ -30436,6 +30564,7 @@
       <c r="M129"/>
       <c r="N129"/>
       <c r="O129"/>
+      <c r="P129"/>
     </row>
     <row r="130">
       <c r="A130" t="n" s="22">
@@ -30467,6 +30596,7 @@
       <c r="M130"/>
       <c r="N130"/>
       <c r="O130"/>
+      <c r="P130"/>
     </row>
     <row r="131">
       <c r="A131" t="n" s="22">
@@ -30498,6 +30628,7 @@
       <c r="M131"/>
       <c r="N131"/>
       <c r="O131"/>
+      <c r="P131"/>
     </row>
     <row r="132">
       <c r="A132" t="n" s="22">
@@ -30531,6 +30662,7 @@
       <c r="M132"/>
       <c r="N132"/>
       <c r="O132"/>
+      <c r="P132"/>
     </row>
     <row r="133">
       <c r="A133" t="n" s="22">
@@ -30564,6 +30696,7 @@
       <c r="M133"/>
       <c r="N133"/>
       <c r="O133"/>
+      <c r="P133"/>
     </row>
     <row r="134">
       <c r="A134" t="n" s="22">
@@ -30595,6 +30728,7 @@
       <c r="M134"/>
       <c r="N134"/>
       <c r="O134"/>
+      <c r="P134"/>
     </row>
     <row r="135">
       <c r="A135" t="n" s="22">
@@ -30626,6 +30760,7 @@
       <c r="M135"/>
       <c r="N135"/>
       <c r="O135"/>
+      <c r="P135"/>
     </row>
     <row r="136">
       <c r="A136" t="n" s="22">
@@ -30659,6 +30794,7 @@
       <c r="M136"/>
       <c r="N136"/>
       <c r="O136"/>
+      <c r="P136"/>
     </row>
     <row r="137">
       <c r="A137" t="n" s="22">
@@ -30692,6 +30828,7 @@
       <c r="M137"/>
       <c r="N137"/>
       <c r="O137"/>
+      <c r="P137"/>
     </row>
     <row r="138">
       <c r="A138" t="n" s="22">
@@ -30723,6 +30860,7 @@
       <c r="M138"/>
       <c r="N138"/>
       <c r="O138"/>
+      <c r="P138"/>
     </row>
     <row r="139">
       <c r="A139" t="n" s="22">
@@ -30754,6 +30892,7 @@
       <c r="M139"/>
       <c r="N139"/>
       <c r="O139"/>
+      <c r="P139"/>
     </row>
     <row r="140">
       <c r="A140" t="n" s="22">
@@ -30787,6 +30926,7 @@
       <c r="M140"/>
       <c r="N140"/>
       <c r="O140"/>
+      <c r="P140"/>
     </row>
     <row r="141">
       <c r="A141" t="n" s="22">
@@ -30820,6 +30960,7 @@
       <c r="M141"/>
       <c r="N141"/>
       <c r="O141"/>
+      <c r="P141"/>
     </row>
     <row r="142">
       <c r="A142" t="n" s="22">
@@ -30851,6 +30992,7 @@
       <c r="M142"/>
       <c r="N142"/>
       <c r="O142"/>
+      <c r="P142"/>
     </row>
     <row r="143">
       <c r="A143" t="n" s="22">
@@ -30882,6 +31024,7 @@
       <c r="M143"/>
       <c r="N143"/>
       <c r="O143"/>
+      <c r="P143"/>
     </row>
     <row r="144">
       <c r="A144" t="n" s="22">
@@ -30913,6 +31056,7 @@
       <c r="M144"/>
       <c r="N144"/>
       <c r="O144"/>
+      <c r="P144"/>
     </row>
     <row r="145">
       <c r="A145" t="n" s="22">
@@ -30944,6 +31088,7 @@
       <c r="M145"/>
       <c r="N145"/>
       <c r="O145"/>
+      <c r="P145"/>
     </row>
     <row r="146">
       <c r="A146" t="n" s="22">
@@ -30975,6 +31120,7 @@
       <c r="M146"/>
       <c r="N146"/>
       <c r="O146"/>
+      <c r="P146"/>
     </row>
     <row r="147">
       <c r="A147" t="n" s="22">
@@ -31006,6 +31152,7 @@
       <c r="M147"/>
       <c r="N147"/>
       <c r="O147"/>
+      <c r="P147"/>
     </row>
     <row r="148">
       <c r="A148" t="n" s="22">
@@ -31037,6 +31184,7 @@
       <c r="M148"/>
       <c r="N148"/>
       <c r="O148"/>
+      <c r="P148"/>
     </row>
     <row r="149">
       <c r="A149" t="n" s="22">
@@ -31068,6 +31216,7 @@
       <c r="M149"/>
       <c r="N149"/>
       <c r="O149"/>
+      <c r="P149"/>
     </row>
     <row r="150">
       <c r="A150" t="n" s="22">
@@ -31099,6 +31248,7 @@
       <c r="M150"/>
       <c r="N150"/>
       <c r="O150"/>
+      <c r="P150"/>
     </row>
     <row r="151">
       <c r="A151" t="n" s="22">
@@ -31132,6 +31282,7 @@
       <c r="M151"/>
       <c r="N151"/>
       <c r="O151"/>
+      <c r="P151"/>
     </row>
     <row r="152">
       <c r="A152" t="n" s="22">
@@ -31165,6 +31316,7 @@
       <c r="M152"/>
       <c r="N152"/>
       <c r="O152"/>
+      <c r="P152"/>
     </row>
     <row r="153">
       <c r="A153" t="n" s="22">
@@ -31198,6 +31350,7 @@
       <c r="M153"/>
       <c r="N153"/>
       <c r="O153"/>
+      <c r="P153"/>
     </row>
     <row r="154">
       <c r="A154" t="n" s="22">
@@ -31229,6 +31382,7 @@
       <c r="M154"/>
       <c r="N154"/>
       <c r="O154"/>
+      <c r="P154"/>
     </row>
     <row r="155">
       <c r="A155" t="n" s="22">
@@ -31260,6 +31414,7 @@
       <c r="M155"/>
       <c r="N155"/>
       <c r="O155"/>
+      <c r="P155"/>
     </row>
     <row r="156">
       <c r="A156" t="n" s="22">
@@ -31291,6 +31446,7 @@
       <c r="M156"/>
       <c r="N156"/>
       <c r="O156"/>
+      <c r="P156"/>
     </row>
     <row r="157">
       <c r="A157" t="n" s="22">
@@ -31324,6 +31480,7 @@
       <c r="M157"/>
       <c r="N157"/>
       <c r="O157"/>
+      <c r="P157"/>
     </row>
     <row r="158">
       <c r="A158" t="n" s="22">
@@ -31357,6 +31514,7 @@
       <c r="M158"/>
       <c r="N158"/>
       <c r="O158"/>
+      <c r="P158"/>
     </row>
     <row r="159">
       <c r="A159" t="n" s="22">
@@ -31388,6 +31546,7 @@
       <c r="M159"/>
       <c r="N159"/>
       <c r="O159"/>
+      <c r="P159"/>
     </row>
     <row r="160">
       <c r="A160" t="n" s="22">
@@ -31419,6 +31578,7 @@
       <c r="M160"/>
       <c r="N160"/>
       <c r="O160"/>
+      <c r="P160"/>
     </row>
     <row r="161">
       <c r="A161" t="n" s="22">
@@ -31450,6 +31610,7 @@
       <c r="M161"/>
       <c r="N161"/>
       <c r="O161"/>
+      <c r="P161"/>
     </row>
     <row r="162">
       <c r="A162" t="n" s="22">
@@ -31483,6 +31644,7 @@
       <c r="M162"/>
       <c r="N162"/>
       <c r="O162"/>
+      <c r="P162"/>
     </row>
     <row r="163">
       <c r="A163" t="n" s="22">
@@ -31516,6 +31678,7 @@
       <c r="M163"/>
       <c r="N163"/>
       <c r="O163"/>
+      <c r="P163"/>
     </row>
     <row r="164">
       <c r="A164" t="n" s="22">
@@ -31547,6 +31710,7 @@
       <c r="M164"/>
       <c r="N164"/>
       <c r="O164"/>
+      <c r="P164"/>
     </row>
     <row r="165">
       <c r="A165" t="n" s="22">
@@ -31578,6 +31742,7 @@
       <c r="M165"/>
       <c r="N165"/>
       <c r="O165"/>
+      <c r="P165"/>
     </row>
     <row r="166">
       <c r="A166" t="n" s="22">
@@ -31609,6 +31774,7 @@
       <c r="M166"/>
       <c r="N166"/>
       <c r="O166"/>
+      <c r="P166"/>
     </row>
     <row r="167">
       <c r="A167" t="n" s="22">
@@ -31640,6 +31806,7 @@
       <c r="M167"/>
       <c r="N167"/>
       <c r="O167"/>
+      <c r="P167"/>
     </row>
     <row r="168">
       <c r="A168" t="n" s="22">
@@ -31671,6 +31838,7 @@
       <c r="M168"/>
       <c r="N168"/>
       <c r="O168"/>
+      <c r="P168"/>
     </row>
     <row r="169">
       <c r="A169" t="n" s="22">
@@ -31702,6 +31870,7 @@
       <c r="M169"/>
       <c r="N169"/>
       <c r="O169"/>
+      <c r="P169"/>
     </row>
     <row r="170">
       <c r="A170" t="n" s="22">
@@ -31733,6 +31902,7 @@
       <c r="M170"/>
       <c r="N170"/>
       <c r="O170"/>
+      <c r="P170"/>
     </row>
     <row r="171">
       <c r="A171" t="n" s="22">
@@ -31764,6 +31934,7 @@
       <c r="M171"/>
       <c r="N171"/>
       <c r="O171"/>
+      <c r="P171"/>
     </row>
     <row r="172">
       <c r="A172" t="n" s="22">
@@ -31795,6 +31966,7 @@
       <c r="M172"/>
       <c r="N172"/>
       <c r="O172"/>
+      <c r="P172"/>
     </row>
     <row r="173">
       <c r="A173" t="n" s="22">
@@ -31826,6 +31998,7 @@
       <c r="M173"/>
       <c r="N173"/>
       <c r="O173"/>
+      <c r="P173"/>
     </row>
     <row r="174">
       <c r="A174" t="n" s="22">
@@ -31859,6 +32032,7 @@
       <c r="M174"/>
       <c r="N174"/>
       <c r="O174"/>
+      <c r="P174"/>
     </row>
     <row r="175">
       <c r="A175" t="n" s="22">
@@ -31892,6 +32066,7 @@
       <c r="M175"/>
       <c r="N175"/>
       <c r="O175"/>
+      <c r="P175"/>
     </row>
     <row r="176">
       <c r="A176" t="n" s="22">
@@ -31923,6 +32098,7 @@
       <c r="M176"/>
       <c r="N176"/>
       <c r="O176"/>
+      <c r="P176"/>
     </row>
     <row r="177">
       <c r="A177" t="n" s="22">
@@ -31954,6 +32130,7 @@
       <c r="M177"/>
       <c r="N177"/>
       <c r="O177"/>
+      <c r="P177"/>
     </row>
     <row r="178">
       <c r="A178" t="n" s="22">
@@ -31985,6 +32162,7 @@
       <c r="M178"/>
       <c r="N178"/>
       <c r="O178"/>
+      <c r="P178"/>
     </row>
     <row r="179">
       <c r="A179" t="n" s="22">
@@ -32018,6 +32196,7 @@
       <c r="M179"/>
       <c r="N179"/>
       <c r="O179"/>
+      <c r="P179"/>
     </row>
     <row r="180">
       <c r="A180" t="n" s="22">
@@ -32051,6 +32230,7 @@
       <c r="M180"/>
       <c r="N180"/>
       <c r="O180"/>
+      <c r="P180"/>
     </row>
     <row r="181">
       <c r="A181" t="n" s="22">
@@ -32082,6 +32262,7 @@
       <c r="M181"/>
       <c r="N181"/>
       <c r="O181"/>
+      <c r="P181"/>
     </row>
     <row r="182">
       <c r="A182" t="n" s="22">
@@ -32113,6 +32294,7 @@
       <c r="M182"/>
       <c r="N182"/>
       <c r="O182"/>
+      <c r="P182"/>
     </row>
     <row r="183">
       <c r="A183" t="n" s="22">
@@ -32144,6 +32326,7 @@
       <c r="M183"/>
       <c r="N183"/>
       <c r="O183"/>
+      <c r="P183"/>
     </row>
     <row r="184">
       <c r="A184" t="n" s="22">
@@ -32177,6 +32360,7 @@
       <c r="M184"/>
       <c r="N184"/>
       <c r="O184"/>
+      <c r="P184"/>
     </row>
     <row r="185">
       <c r="A185" t="n" s="22">
@@ -32210,6 +32394,7 @@
       <c r="M185"/>
       <c r="N185"/>
       <c r="O185"/>
+      <c r="P185"/>
     </row>
     <row r="186">
       <c r="A186" t="n" s="22">
@@ -32241,6 +32426,7 @@
       <c r="M186"/>
       <c r="N186"/>
       <c r="O186"/>
+      <c r="P186"/>
     </row>
     <row r="187">
       <c r="A187" t="n" s="22">
@@ -32272,6 +32458,7 @@
       <c r="M187"/>
       <c r="N187"/>
       <c r="O187"/>
+      <c r="P187"/>
     </row>
     <row r="188">
       <c r="A188" t="n" s="22">
@@ -32303,6 +32490,7 @@
       <c r="M188"/>
       <c r="N188"/>
       <c r="O188"/>
+      <c r="P188"/>
     </row>
     <row r="189">
       <c r="A189" t="n" s="22">
@@ -32334,6 +32522,7 @@
       <c r="M189"/>
       <c r="N189"/>
       <c r="O189"/>
+      <c r="P189"/>
     </row>
     <row r="190">
       <c r="A190" t="n" s="22">
@@ -32365,6 +32554,7 @@
       <c r="M190"/>
       <c r="N190"/>
       <c r="O190"/>
+      <c r="P190"/>
     </row>
     <row r="191">
       <c r="A191" t="n" s="22">
@@ -32396,6 +32586,7 @@
       <c r="M191"/>
       <c r="N191"/>
       <c r="O191"/>
+      <c r="P191"/>
     </row>
     <row r="192">
       <c r="A192" t="n" s="22">
@@ -32427,6 +32618,7 @@
       <c r="M192"/>
       <c r="N192"/>
       <c r="O192"/>
+      <c r="P192"/>
     </row>
     <row r="193">
       <c r="A193" t="n" s="22">
@@ -32458,6 +32650,7 @@
       <c r="M193"/>
       <c r="N193"/>
       <c r="O193"/>
+      <c r="P193"/>
     </row>
     <row r="194">
       <c r="A194" t="n" s="22">
@@ -32489,6 +32682,7 @@
       <c r="M194"/>
       <c r="N194"/>
       <c r="O194"/>
+      <c r="P194"/>
     </row>
     <row r="195">
       <c r="A195" t="n" s="22">
@@ -32522,6 +32716,7 @@
       <c r="M195"/>
       <c r="N195"/>
       <c r="O195"/>
+      <c r="P195"/>
     </row>
     <row r="196">
       <c r="A196" t="n" s="22">
@@ -32555,6 +32750,7 @@
       <c r="M196"/>
       <c r="N196"/>
       <c r="O196"/>
+      <c r="P196"/>
     </row>
     <row r="197">
       <c r="A197" t="n" s="22">
@@ -32588,6 +32784,7 @@
       <c r="M197"/>
       <c r="N197"/>
       <c r="O197"/>
+      <c r="P197"/>
     </row>
     <row r="198">
       <c r="A198" t="n" s="22">
@@ -32619,6 +32816,7 @@
       <c r="M198"/>
       <c r="N198"/>
       <c r="O198"/>
+      <c r="P198"/>
     </row>
     <row r="199">
       <c r="A199" t="n" s="22">
@@ -32650,6 +32848,7 @@
       <c r="M199"/>
       <c r="N199"/>
       <c r="O199"/>
+      <c r="P199"/>
     </row>
     <row r="200">
       <c r="A200" t="n" s="22">
@@ -32681,6 +32880,7 @@
       <c r="M200"/>
       <c r="N200"/>
       <c r="O200"/>
+      <c r="P200"/>
     </row>
     <row r="201">
       <c r="A201" t="n" s="22">
@@ -32714,6 +32914,7 @@
       <c r="M201"/>
       <c r="N201"/>
       <c r="O201"/>
+      <c r="P201"/>
     </row>
     <row r="202">
       <c r="A202" t="n" s="22">
@@ -32747,6 +32948,7 @@
       <c r="M202"/>
       <c r="N202"/>
       <c r="O202"/>
+      <c r="P202"/>
     </row>
     <row r="203">
       <c r="A203" t="n" s="22">
@@ -32778,6 +32980,7 @@
       <c r="M203"/>
       <c r="N203"/>
       <c r="O203"/>
+      <c r="P203"/>
     </row>
     <row r="204">
       <c r="A204" t="n" s="22">
@@ -32809,6 +33012,7 @@
       <c r="M204"/>
       <c r="N204"/>
       <c r="O204"/>
+      <c r="P204"/>
     </row>
     <row r="205">
       <c r="A205" t="n" s="22">
@@ -32840,6 +33044,7 @@
       <c r="M205"/>
       <c r="N205"/>
       <c r="O205"/>
+      <c r="P205"/>
     </row>
     <row r="206">
       <c r="A206" t="n" s="22">
@@ -32873,6 +33078,7 @@
       <c r="M206"/>
       <c r="N206"/>
       <c r="O206"/>
+      <c r="P206"/>
     </row>
     <row r="207">
       <c r="A207" t="n" s="22">
@@ -32906,6 +33112,7 @@
       <c r="M207"/>
       <c r="N207"/>
       <c r="O207"/>
+      <c r="P207"/>
     </row>
     <row r="208">
       <c r="A208" t="n" s="22">
@@ -32937,6 +33144,7 @@
       <c r="M208"/>
       <c r="N208"/>
       <c r="O208"/>
+      <c r="P208"/>
     </row>
     <row r="209">
       <c r="A209" t="n" s="22">
@@ -32968,6 +33176,7 @@
       <c r="M209"/>
       <c r="N209"/>
       <c r="O209"/>
+      <c r="P209"/>
     </row>
     <row r="210">
       <c r="A210" t="n" s="22">
@@ -32999,6 +33208,7 @@
       <c r="M210"/>
       <c r="N210"/>
       <c r="O210"/>
+      <c r="P210"/>
     </row>
     <row r="211">
       <c r="A211" t="n" s="22">
@@ -33030,6 +33240,7 @@
       <c r="M211"/>
       <c r="N211"/>
       <c r="O211"/>
+      <c r="P211"/>
     </row>
     <row r="212">
       <c r="A212" t="n" s="22">
@@ -33061,6 +33272,7 @@
       <c r="M212"/>
       <c r="N212"/>
       <c r="O212"/>
+      <c r="P212"/>
     </row>
     <row r="213">
       <c r="A213" t="n" s="22">
@@ -33092,6 +33304,7 @@
       <c r="M213"/>
       <c r="N213"/>
       <c r="O213"/>
+      <c r="P213"/>
     </row>
     <row r="214">
       <c r="A214" t="n" s="22">
@@ -33123,6 +33336,7 @@
       <c r="M214"/>
       <c r="N214"/>
       <c r="O214"/>
+      <c r="P214"/>
     </row>
     <row r="215">
       <c r="A215" t="n" s="22">
@@ -33154,6 +33368,7 @@
       <c r="M215"/>
       <c r="N215"/>
       <c r="O215"/>
+      <c r="P215"/>
     </row>
     <row r="216">
       <c r="A216" t="n" s="22">
@@ -33185,6 +33400,7 @@
       <c r="M216"/>
       <c r="N216"/>
       <c r="O216"/>
+      <c r="P216"/>
     </row>
     <row r="217">
       <c r="A217" t="n" s="22">
@@ -33216,6 +33432,7 @@
       <c r="M217"/>
       <c r="N217"/>
       <c r="O217"/>
+      <c r="P217"/>
     </row>
     <row r="218">
       <c r="A218" t="n" s="22">
@@ -33249,6 +33466,7 @@
       <c r="M218"/>
       <c r="N218"/>
       <c r="O218"/>
+      <c r="P218"/>
     </row>
     <row r="219">
       <c r="A219" t="n" s="22">
@@ -33282,6 +33500,7 @@
       <c r="M219"/>
       <c r="N219"/>
       <c r="O219"/>
+      <c r="P219"/>
     </row>
     <row r="220">
       <c r="A220" t="n" s="22">
@@ -33313,6 +33532,7 @@
       <c r="M220"/>
       <c r="N220"/>
       <c r="O220"/>
+      <c r="P220"/>
     </row>
     <row r="221">
       <c r="A221" t="n" s="22">
@@ -33344,6 +33564,7 @@
       <c r="M221"/>
       <c r="N221"/>
       <c r="O221"/>
+      <c r="P221"/>
     </row>
     <row r="222">
       <c r="A222" t="n" s="22">
@@ -33375,6 +33596,7 @@
       <c r="M222"/>
       <c r="N222"/>
       <c r="O222"/>
+      <c r="P222"/>
     </row>
     <row r="223">
       <c r="A223" t="n" s="22">
@@ -33408,6 +33630,7 @@
       <c r="M223"/>
       <c r="N223"/>
       <c r="O223"/>
+      <c r="P223"/>
     </row>
     <row r="224">
       <c r="A224" t="n" s="22">
@@ -33441,6 +33664,7 @@
       <c r="M224"/>
       <c r="N224"/>
       <c r="O224"/>
+      <c r="P224"/>
     </row>
     <row r="225">
       <c r="A225" t="n" s="22">
@@ -33472,6 +33696,7 @@
       <c r="M225"/>
       <c r="N225"/>
       <c r="O225"/>
+      <c r="P225"/>
     </row>
     <row r="226">
       <c r="A226" t="n" s="22">
@@ -33503,6 +33728,7 @@
       <c r="M226"/>
       <c r="N226"/>
       <c r="O226"/>
+      <c r="P226"/>
     </row>
     <row r="227">
       <c r="A227" t="n" s="22">
@@ -33534,6 +33760,7 @@
       <c r="M227"/>
       <c r="N227"/>
       <c r="O227"/>
+      <c r="P227"/>
     </row>
     <row r="228">
       <c r="A228" t="n" s="22">
@@ -33567,6 +33794,7 @@
       <c r="M228"/>
       <c r="N228"/>
       <c r="O228"/>
+      <c r="P228"/>
     </row>
     <row r="229">
       <c r="A229" t="n" s="22">
@@ -33600,6 +33828,7 @@
       <c r="M229"/>
       <c r="N229"/>
       <c r="O229"/>
+      <c r="P229"/>
     </row>
     <row r="230">
       <c r="A230" t="n" s="22">
@@ -33631,6 +33860,7 @@
       <c r="M230"/>
       <c r="N230"/>
       <c r="O230"/>
+      <c r="P230"/>
     </row>
     <row r="231">
       <c r="A231" t="n" s="22">
@@ -33662,6 +33892,7 @@
       <c r="M231"/>
       <c r="N231"/>
       <c r="O231"/>
+      <c r="P231"/>
     </row>
     <row r="232">
       <c r="A232" t="n" s="22">
@@ -33693,6 +33924,7 @@
       <c r="M232"/>
       <c r="N232"/>
       <c r="O232"/>
+      <c r="P232"/>
     </row>
     <row r="233">
       <c r="A233" t="n" s="22">
@@ -33724,6 +33956,7 @@
       <c r="M233"/>
       <c r="N233"/>
       <c r="O233"/>
+      <c r="P233"/>
     </row>
     <row r="234">
       <c r="A234" t="n" s="22">
@@ -33755,6 +33988,7 @@
       <c r="M234"/>
       <c r="N234"/>
       <c r="O234"/>
+      <c r="P234"/>
     </row>
     <row r="235">
       <c r="A235" t="n" s="22">
@@ -33786,6 +34020,7 @@
       <c r="M235"/>
       <c r="N235"/>
       <c r="O235"/>
+      <c r="P235"/>
     </row>
     <row r="236">
       <c r="A236" t="n" s="22">
@@ -33817,6 +34052,7 @@
       <c r="M236"/>
       <c r="N236"/>
       <c r="O236"/>
+      <c r="P236"/>
     </row>
     <row r="237">
       <c r="A237" t="n" s="22">
@@ -33848,6 +34084,7 @@
       <c r="M237"/>
       <c r="N237"/>
       <c r="O237"/>
+      <c r="P237"/>
     </row>
     <row r="238">
       <c r="A238" t="n" s="22">
@@ -33879,6 +34116,7 @@
       <c r="M238"/>
       <c r="N238"/>
       <c r="O238"/>
+      <c r="P238"/>
     </row>
     <row r="239">
       <c r="A239" t="n" s="22">
@@ -33910,6 +34148,7 @@
       <c r="M239"/>
       <c r="N239"/>
       <c r="O239"/>
+      <c r="P239"/>
     </row>
     <row r="240">
       <c r="A240" t="n" s="22">
@@ -33943,6 +34182,7 @@
       </c>
       <c r="N240"/>
       <c r="O240"/>
+      <c r="P240"/>
     </row>
     <row r="241">
       <c r="A241" t="n" s="22">
@@ -33974,6 +34214,7 @@
       <c r="M241"/>
       <c r="N241"/>
       <c r="O241"/>
+      <c r="P241"/>
     </row>
     <row r="242">
       <c r="A242" t="n" s="22">
@@ -34007,6 +34248,7 @@
       </c>
       <c r="N242"/>
       <c r="O242"/>
+      <c r="P242"/>
     </row>
     <row r="243">
       <c r="A243" t="n" s="22">
@@ -34040,6 +34282,7 @@
       <c r="M243"/>
       <c r="N243"/>
       <c r="O243"/>
+      <c r="P243"/>
     </row>
     <row r="244">
       <c r="A244" t="n" s="22">
@@ -34075,6 +34318,7 @@
       <c r="M244"/>
       <c r="N244"/>
       <c r="O244"/>
+      <c r="P244"/>
     </row>
     <row r="245">
       <c r="A245" t="n" s="22">
@@ -34106,6 +34350,7 @@
       <c r="M245"/>
       <c r="N245"/>
       <c r="O245"/>
+      <c r="P245"/>
     </row>
     <row r="246">
       <c r="A246" t="n" s="22">
@@ -34137,6 +34382,7 @@
       <c r="M246"/>
       <c r="N246"/>
       <c r="O246"/>
+      <c r="P246"/>
     </row>
     <row r="247">
       <c r="A247" t="n" s="22">
@@ -34168,6 +34414,7 @@
       <c r="M247"/>
       <c r="N247"/>
       <c r="O247"/>
+      <c r="P247"/>
     </row>
     <row r="248">
       <c r="A248" t="n" s="22">
@@ -34201,6 +34448,7 @@
       <c r="M248"/>
       <c r="N248"/>
       <c r="O248"/>
+      <c r="P248"/>
     </row>
     <row r="249">
       <c r="A249" t="n" s="22">
@@ -34232,6 +34480,7 @@
       <c r="M249"/>
       <c r="N249"/>
       <c r="O249"/>
+      <c r="P249"/>
     </row>
     <row r="250">
       <c r="A250" t="n" s="22">
@@ -34263,6 +34512,7 @@
       <c r="M250"/>
       <c r="N250"/>
       <c r="O250"/>
+      <c r="P250"/>
     </row>
     <row r="251">
       <c r="A251" t="n" s="22">
@@ -34294,6 +34544,7 @@
       <c r="M251"/>
       <c r="N251"/>
       <c r="O251"/>
+      <c r="P251"/>
     </row>
     <row r="252">
       <c r="A252" t="n" s="22">
@@ -34325,6 +34576,7 @@
       <c r="M252"/>
       <c r="N252"/>
       <c r="O252"/>
+      <c r="P252"/>
     </row>
     <row r="253">
       <c r="A253" t="n" s="22">
@@ -34356,6 +34608,7 @@
       <c r="M253"/>
       <c r="N253"/>
       <c r="O253"/>
+      <c r="P253"/>
     </row>
     <row r="254">
       <c r="A254" t="n" s="22">
@@ -34385,6 +34638,7 @@
       <c r="M254"/>
       <c r="N254"/>
       <c r="O254"/>
+      <c r="P254"/>
     </row>
     <row r="255">
       <c r="A255" t="n" s="22">
@@ -34414,6 +34668,7 @@
       <c r="M255"/>
       <c r="N255"/>
       <c r="O255"/>
+      <c r="P255"/>
     </row>
     <row r="256">
       <c r="A256" t="n" s="22">
@@ -34443,6 +34698,7 @@
       <c r="M256"/>
       <c r="N256"/>
       <c r="O256"/>
+      <c r="P256"/>
     </row>
     <row r="257">
       <c r="A257" t="n" s="22">
@@ -34450,16 +34706,16 @@
       </c>
       <c r="B257"/>
       <c r="C257" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="D257" t="s">
-        <v>774</v>
+        <v>768</v>
       </c>
       <c r="E257" t="s">
-        <v>313</v>
+        <v>443</v>
       </c>
       <c r="F257" t="s">
-        <v>666</v>
+        <v>658</v>
       </c>
       <c r="G257"/>
       <c r="H257"/>
@@ -34468,12 +34724,15 @@
         <v>1.0</v>
       </c>
       <c r="K257" t="s">
-        <v>1257</v>
+        <v>1226</v>
       </c>
       <c r="L257"/>
       <c r="M257"/>
       <c r="N257"/>
       <c r="O257"/>
+      <c r="P257" t="s">
+        <v>660</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="n" s="22">
@@ -34490,21 +34749,22 @@
         <v>313</v>
       </c>
       <c r="F258" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="G258"/>
       <c r="H258"/>
       <c r="I258"/>
       <c r="J258" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K258" t="s">
-        <v>1226</v>
+        <v>1257</v>
       </c>
       <c r="L258"/>
       <c r="M258"/>
       <c r="N258"/>
       <c r="O258"/>
+      <c r="P258"/>
     </row>
     <row r="259">
       <c r="A259" t="n" s="22">
@@ -34521,13 +34781,13 @@
         <v>313</v>
       </c>
       <c r="F259" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G259"/>
       <c r="H259"/>
       <c r="I259"/>
       <c r="J259" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K259" t="s">
         <v>1226</v>
@@ -34536,6 +34796,7 @@
       <c r="M259"/>
       <c r="N259"/>
       <c r="O259"/>
+      <c r="P259"/>
     </row>
     <row r="260">
       <c r="A260" t="n" s="22">
@@ -34546,19 +34807,19 @@
         <v>80</v>
       </c>
       <c r="D260" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="E260" t="s">
         <v>313</v>
       </c>
       <c r="F260" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="G260"/>
       <c r="H260"/>
       <c r="I260"/>
       <c r="J260" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K260" t="s">
         <v>1226</v>
@@ -34567,6 +34828,7 @@
       <c r="M260"/>
       <c r="N260"/>
       <c r="O260"/>
+      <c r="P260"/>
     </row>
     <row r="261">
       <c r="A261" t="n" s="22">
@@ -34583,13 +34845,13 @@
         <v>313</v>
       </c>
       <c r="F261" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="G261"/>
       <c r="H261"/>
       <c r="I261"/>
       <c r="J261" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K261" t="s">
         <v>1226</v>
@@ -34598,6 +34860,7 @@
       <c r="M261"/>
       <c r="N261"/>
       <c r="O261"/>
+      <c r="P261"/>
     </row>
     <row r="262">
       <c r="A262" t="n" s="22">
@@ -34614,13 +34877,13 @@
         <v>313</v>
       </c>
       <c r="F262" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G262"/>
       <c r="H262"/>
       <c r="I262"/>
       <c r="J262" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K262" t="s">
         <v>1226</v>
@@ -34629,6 +34892,7 @@
       <c r="M262"/>
       <c r="N262"/>
       <c r="O262"/>
+      <c r="P262"/>
     </row>
     <row r="263">
       <c r="A263" t="n" s="22">
@@ -34636,22 +34900,22 @@
       </c>
       <c r="B263"/>
       <c r="C263" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="D263" t="s">
-        <v>768</v>
+        <v>776</v>
       </c>
       <c r="E263" t="s">
-        <v>99</v>
+        <v>313</v>
       </c>
       <c r="F263" t="s">
-        <v>433</v>
+        <v>670</v>
       </c>
       <c r="G263"/>
       <c r="H263"/>
       <c r="I263"/>
       <c r="J263" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K263" t="s">
         <v>1226</v>
@@ -34660,6 +34924,7 @@
       <c r="M263"/>
       <c r="N263"/>
       <c r="O263"/>
+      <c r="P263"/>
     </row>
     <row r="264">
       <c r="A264" t="n" s="22">
@@ -34670,7 +34935,7 @@
         <v>98</v>
       </c>
       <c r="D264" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="E264" t="s">
         <v>99</v>
@@ -34682,7 +34947,7 @@
       <c r="H264"/>
       <c r="I264"/>
       <c r="J264" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K264" t="s">
         <v>1226</v>
@@ -34691,29 +34956,30 @@
       <c r="M264"/>
       <c r="N264"/>
       <c r="O264"/>
+      <c r="P264"/>
     </row>
     <row r="265">
       <c r="A265" t="n" s="22">
-        <v>43836.0</v>
+        <v>43101.0</v>
       </c>
       <c r="B265"/>
       <c r="C265" t="s">
-        <v>63</v>
+        <v>98</v>
       </c>
       <c r="D265" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="E265" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
       <c r="F265" t="s">
-        <v>68</v>
+        <v>433</v>
       </c>
       <c r="G265"/>
       <c r="H265"/>
       <c r="I265"/>
       <c r="J265" t="n">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="K265" t="s">
         <v>1226</v>
@@ -34722,6 +34988,7 @@
       <c r="M265"/>
       <c r="N265"/>
       <c r="O265"/>
+      <c r="P265"/>
     </row>
     <row r="266">
       <c r="A266" t="n" s="22">
@@ -34738,13 +35005,13 @@
         <v>73</v>
       </c>
       <c r="F266" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G266"/>
       <c r="H266"/>
       <c r="I266"/>
       <c r="J266" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K266" t="s">
         <v>1226</v>
@@ -34753,6 +35020,7 @@
       <c r="M266"/>
       <c r="N266"/>
       <c r="O266"/>
+      <c r="P266"/>
     </row>
     <row r="267">
       <c r="A267" t="n" s="22">
@@ -34769,13 +35037,13 @@
         <v>73</v>
       </c>
       <c r="F267" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G267"/>
       <c r="H267"/>
       <c r="I267"/>
       <c r="J267" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K267" t="s">
         <v>1226</v>
@@ -34784,6 +35052,7 @@
       <c r="M267"/>
       <c r="N267"/>
       <c r="O267"/>
+      <c r="P267"/>
     </row>
     <row r="268">
       <c r="A268" t="n" s="22">
@@ -34800,13 +35069,13 @@
         <v>73</v>
       </c>
       <c r="F268" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G268"/>
       <c r="H268"/>
       <c r="I268"/>
       <c r="J268" t="n">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="K268" t="s">
         <v>1226</v>
@@ -34815,6 +35084,7 @@
       <c r="M268"/>
       <c r="N268"/>
       <c r="O268"/>
+      <c r="P268"/>
     </row>
     <row r="269">
       <c r="A269" t="n" s="22">
@@ -34828,16 +35098,16 @@
         <v>768</v>
       </c>
       <c r="E269" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F269" t="s">
-        <v>68</v>
+        <v>684</v>
       </c>
       <c r="G269"/>
       <c r="H269"/>
       <c r="I269"/>
       <c r="J269" t="n">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="K269" t="s">
         <v>1226</v>
@@ -34846,6 +35116,7 @@
       <c r="M269"/>
       <c r="N269"/>
       <c r="O269"/>
+      <c r="P269"/>
     </row>
     <row r="270">
       <c r="A270" t="n" s="22">
@@ -34862,13 +35133,13 @@
         <v>72</v>
       </c>
       <c r="F270" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G270"/>
       <c r="H270"/>
       <c r="I270"/>
       <c r="J270" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="K270" t="s">
         <v>1226</v>
@@ -34877,6 +35148,7 @@
       <c r="M270"/>
       <c r="N270"/>
       <c r="O270"/>
+      <c r="P270"/>
     </row>
     <row r="271">
       <c r="A271" t="n" s="22">
@@ -34893,13 +35165,13 @@
         <v>72</v>
       </c>
       <c r="F271" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G271"/>
       <c r="H271"/>
       <c r="I271"/>
       <c r="J271" t="n">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="K271" t="s">
         <v>1226</v>
@@ -34908,6 +35180,7 @@
       <c r="M271"/>
       <c r="N271"/>
       <c r="O271"/>
+      <c r="P271"/>
     </row>
     <row r="272">
       <c r="A272" t="n" s="22">
@@ -34924,13 +35197,13 @@
         <v>72</v>
       </c>
       <c r="F272" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G272"/>
       <c r="H272"/>
       <c r="I272"/>
       <c r="J272" t="n">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="K272" t="s">
         <v>1226</v>
@@ -34939,6 +35212,7 @@
       <c r="M272"/>
       <c r="N272"/>
       <c r="O272"/>
+      <c r="P272"/>
     </row>
     <row r="273">
       <c r="A273" t="n" s="22">
@@ -34949,19 +35223,19 @@
         <v>63</v>
       </c>
       <c r="D273" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="E273" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F273" t="s">
-        <v>68</v>
+        <v>684</v>
       </c>
       <c r="G273"/>
       <c r="H273"/>
       <c r="I273"/>
       <c r="J273" t="n">
-        <v>1.0</v>
+        <v>8.0</v>
       </c>
       <c r="K273" t="s">
         <v>1226</v>
@@ -34970,6 +35244,7 @@
       <c r="M273"/>
       <c r="N273"/>
       <c r="O273"/>
+      <c r="P273"/>
     </row>
     <row r="274">
       <c r="A274" t="n" s="22">
@@ -34986,13 +35261,13 @@
         <v>73</v>
       </c>
       <c r="F274" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G274"/>
       <c r="H274"/>
       <c r="I274"/>
       <c r="J274" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K274" t="s">
         <v>1226</v>
@@ -35001,6 +35276,7 @@
       <c r="M274"/>
       <c r="N274"/>
       <c r="O274"/>
+      <c r="P274"/>
     </row>
     <row r="275">
       <c r="A275" t="n" s="22">
@@ -35017,13 +35293,13 @@
         <v>73</v>
       </c>
       <c r="F275" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G275"/>
       <c r="H275"/>
       <c r="I275"/>
       <c r="J275" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K275" t="s">
         <v>1226</v>
@@ -35032,6 +35308,7 @@
       <c r="M275"/>
       <c r="N275"/>
       <c r="O275"/>
+      <c r="P275"/>
     </row>
     <row r="276">
       <c r="A276" t="n" s="22">
@@ -35048,13 +35325,13 @@
         <v>73</v>
       </c>
       <c r="F276" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G276"/>
       <c r="H276"/>
       <c r="I276"/>
       <c r="J276" t="n">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="K276" t="s">
         <v>1226</v>
@@ -35063,6 +35340,7 @@
       <c r="M276"/>
       <c r="N276"/>
       <c r="O276"/>
+      <c r="P276"/>
     </row>
     <row r="277">
       <c r="A277" t="n" s="22">
@@ -35076,16 +35354,16 @@
         <v>770</v>
       </c>
       <c r="E277" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F277" t="s">
-        <v>68</v>
+        <v>684</v>
       </c>
       <c r="G277"/>
       <c r="H277"/>
       <c r="I277"/>
       <c r="J277" t="n">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="K277" t="s">
         <v>1226</v>
@@ -35094,6 +35372,7 @@
       <c r="M277"/>
       <c r="N277"/>
       <c r="O277"/>
+      <c r="P277"/>
     </row>
     <row r="278">
       <c r="A278" t="n" s="22">
@@ -35110,13 +35389,13 @@
         <v>72</v>
       </c>
       <c r="F278" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G278"/>
       <c r="H278"/>
       <c r="I278"/>
       <c r="J278" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="K278" t="s">
         <v>1226</v>
@@ -35125,6 +35404,7 @@
       <c r="M278"/>
       <c r="N278"/>
       <c r="O278"/>
+      <c r="P278"/>
     </row>
     <row r="279">
       <c r="A279" t="n" s="22">
@@ -35141,13 +35421,13 @@
         <v>72</v>
       </c>
       <c r="F279" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G279"/>
       <c r="H279"/>
       <c r="I279"/>
       <c r="J279" t="n">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="K279" t="s">
         <v>1226</v>
@@ -35156,6 +35436,7 @@
       <c r="M279"/>
       <c r="N279"/>
       <c r="O279"/>
+      <c r="P279"/>
     </row>
     <row r="280">
       <c r="A280" t="n" s="22">
@@ -35172,13 +35453,13 @@
         <v>72</v>
       </c>
       <c r="F280" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G280"/>
       <c r="H280"/>
       <c r="I280"/>
       <c r="J280" t="n">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="K280" t="s">
         <v>1226</v>
@@ -35187,6 +35468,7 @@
       <c r="M280"/>
       <c r="N280"/>
       <c r="O280"/>
+      <c r="P280"/>
     </row>
     <row r="281">
       <c r="A281" t="n" s="22">
@@ -35200,16 +35482,16 @@
         <v>770</v>
       </c>
       <c r="E281" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F281" t="s">
-        <v>68</v>
+        <v>684</v>
       </c>
       <c r="G281"/>
       <c r="H281"/>
       <c r="I281"/>
       <c r="J281" t="n">
-        <v>5.0</v>
+        <v>8.0</v>
       </c>
       <c r="K281" t="s">
         <v>1226</v>
@@ -35218,6 +35500,7 @@
       <c r="M281"/>
       <c r="N281"/>
       <c r="O281"/>
+      <c r="P281"/>
     </row>
     <row r="282">
       <c r="A282" t="n" s="22">
@@ -35234,13 +35517,13 @@
         <v>74</v>
       </c>
       <c r="F282" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G282"/>
       <c r="H282"/>
       <c r="I282"/>
       <c r="J282" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="K282" t="s">
         <v>1226</v>
@@ -35249,6 +35532,7 @@
       <c r="M282"/>
       <c r="N282"/>
       <c r="O282"/>
+      <c r="P282"/>
     </row>
     <row r="283">
       <c r="A283" t="n" s="22">
@@ -35265,13 +35549,13 @@
         <v>74</v>
       </c>
       <c r="F283" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G283"/>
       <c r="H283"/>
       <c r="I283"/>
       <c r="J283" t="n">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="K283" t="s">
         <v>1226</v>
@@ -35280,6 +35564,7 @@
       <c r="M283"/>
       <c r="N283"/>
       <c r="O283"/>
+      <c r="P283"/>
     </row>
     <row r="284">
       <c r="A284" t="n" s="22">
@@ -35296,13 +35581,13 @@
         <v>74</v>
       </c>
       <c r="F284" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G284"/>
       <c r="H284"/>
       <c r="I284"/>
       <c r="J284" t="n">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="K284" t="s">
         <v>1226</v>
@@ -35311,6 +35596,39 @@
       <c r="M284"/>
       <c r="N284"/>
       <c r="O284"/>
+      <c r="P284"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="n" s="22">
+        <v>43836.0</v>
+      </c>
+      <c r="B285"/>
+      <c r="C285" t="s">
+        <v>63</v>
+      </c>
+      <c r="D285" t="s">
+        <v>770</v>
+      </c>
+      <c r="E285" t="s">
+        <v>74</v>
+      </c>
+      <c r="F285" t="s">
+        <v>684</v>
+      </c>
+      <c r="G285"/>
+      <c r="H285"/>
+      <c r="I285"/>
+      <c r="J285" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="K285" t="s">
+        <v>1226</v>
+      </c>
+      <c r="L285"/>
+      <c r="M285"/>
+      <c r="N285"/>
+      <c r="O285"/>
+      <c r="P285"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
CCD-8328: Updating with master
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16264" uniqueCount="1564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16271" uniqueCount="1564">
   <si>
     <t>SearchInputFields</t>
   </si>
@@ -26606,7 +26606,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O284"/>
+  <dimension ref="A1:P285"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -26661,6 +26661,9 @@
       <c r="O3" t="s">
         <v>1225</v>
       </c>
+      <c r="P3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n" s="22">
@@ -26692,6 +26695,7 @@
       <c r="M4"/>
       <c r="N4"/>
       <c r="O4"/>
+      <c r="P4"/>
     </row>
     <row r="5">
       <c r="A5" t="n" s="22">
@@ -26723,6 +26727,7 @@
       <c r="M5"/>
       <c r="N5"/>
       <c r="O5"/>
+      <c r="P5"/>
     </row>
     <row r="6">
       <c r="A6" t="n" s="22">
@@ -26754,6 +26759,7 @@
       <c r="M6"/>
       <c r="N6"/>
       <c r="O6"/>
+      <c r="P6"/>
     </row>
     <row r="7">
       <c r="A7" t="n" s="22">
@@ -26785,6 +26791,7 @@
       <c r="M7"/>
       <c r="N7"/>
       <c r="O7"/>
+      <c r="P7"/>
     </row>
     <row r="8">
       <c r="A8" t="n" s="22">
@@ -26816,6 +26823,7 @@
       <c r="M8"/>
       <c r="N8"/>
       <c r="O8"/>
+      <c r="P8"/>
     </row>
     <row r="9">
       <c r="A9" t="n" s="22">
@@ -26847,6 +26855,7 @@
       <c r="M9"/>
       <c r="N9"/>
       <c r="O9"/>
+      <c r="P9"/>
     </row>
     <row r="10">
       <c r="A10" t="n" s="22">
@@ -26878,6 +26887,7 @@
       <c r="M10"/>
       <c r="N10"/>
       <c r="O10"/>
+      <c r="P10"/>
     </row>
     <row r="11">
       <c r="A11" t="n" s="22">
@@ -26909,6 +26919,7 @@
       <c r="M11"/>
       <c r="N11"/>
       <c r="O11"/>
+      <c r="P11"/>
     </row>
     <row r="12">
       <c r="A12" t="n" s="22">
@@ -26940,6 +26951,7 @@
       <c r="M12"/>
       <c r="N12"/>
       <c r="O12"/>
+      <c r="P12"/>
     </row>
     <row r="13">
       <c r="A13" t="n" s="22">
@@ -26971,6 +26983,7 @@
       <c r="M13"/>
       <c r="N13"/>
       <c r="O13"/>
+      <c r="P13"/>
     </row>
     <row r="14">
       <c r="A14" t="n" s="22">
@@ -27004,6 +27017,7 @@
       <c r="M14"/>
       <c r="N14"/>
       <c r="O14"/>
+      <c r="P14"/>
     </row>
     <row r="15">
       <c r="A15" t="n" s="22">
@@ -27039,6 +27053,7 @@
       <c r="M15"/>
       <c r="N15"/>
       <c r="O15"/>
+      <c r="P15"/>
     </row>
     <row r="16">
       <c r="A16" t="n" s="22">
@@ -27070,6 +27085,7 @@
       <c r="M16"/>
       <c r="N16"/>
       <c r="O16"/>
+      <c r="P16"/>
     </row>
     <row r="17">
       <c r="A17" t="n" s="22">
@@ -27101,6 +27117,7 @@
       <c r="M17"/>
       <c r="N17"/>
       <c r="O17"/>
+      <c r="P17"/>
     </row>
     <row r="18">
       <c r="A18" t="n" s="22">
@@ -27132,6 +27149,7 @@
       <c r="M18"/>
       <c r="N18"/>
       <c r="O18"/>
+      <c r="P18"/>
     </row>
     <row r="19">
       <c r="A19" t="n" s="22">
@@ -27165,6 +27183,7 @@
       <c r="M19"/>
       <c r="N19"/>
       <c r="O19"/>
+      <c r="P19"/>
     </row>
     <row r="20">
       <c r="A20" t="n" s="22">
@@ -27196,6 +27215,7 @@
       <c r="M20"/>
       <c r="N20"/>
       <c r="O20"/>
+      <c r="P20"/>
     </row>
     <row r="21">
       <c r="A21" t="n" s="22">
@@ -27233,6 +27253,7 @@
       <c r="O21" t="s">
         <v>1242</v>
       </c>
+      <c r="P21"/>
     </row>
     <row r="22">
       <c r="A22" t="n" s="22">
@@ -27266,6 +27287,7 @@
       <c r="M22"/>
       <c r="N22"/>
       <c r="O22"/>
+      <c r="P22"/>
     </row>
     <row r="23">
       <c r="A23" t="n" s="22">
@@ -27297,6 +27319,7 @@
       <c r="M23"/>
       <c r="N23"/>
       <c r="O23"/>
+      <c r="P23"/>
     </row>
     <row r="24">
       <c r="A24" t="n" s="22">
@@ -27328,6 +27351,7 @@
       <c r="M24"/>
       <c r="N24"/>
       <c r="O24"/>
+      <c r="P24"/>
     </row>
     <row r="25">
       <c r="A25" t="n" s="22">
@@ -27361,6 +27385,7 @@
       <c r="M25"/>
       <c r="N25"/>
       <c r="O25"/>
+      <c r="P25"/>
     </row>
     <row r="26">
       <c r="A26" t="n" s="22">
@@ -27392,6 +27417,7 @@
       <c r="M26"/>
       <c r="N26"/>
       <c r="O26"/>
+      <c r="P26"/>
     </row>
     <row r="27">
       <c r="A27" t="n" s="22">
@@ -27423,6 +27449,7 @@
       <c r="M27"/>
       <c r="N27"/>
       <c r="O27"/>
+      <c r="P27"/>
     </row>
     <row r="28">
       <c r="A28" t="n" s="22">
@@ -27454,6 +27481,7 @@
       <c r="M28"/>
       <c r="N28"/>
       <c r="O28"/>
+      <c r="P28"/>
     </row>
     <row r="29">
       <c r="A29" t="n" s="22">
@@ -27485,6 +27513,7 @@
       <c r="M29"/>
       <c r="N29"/>
       <c r="O29"/>
+      <c r="P29"/>
     </row>
     <row r="30">
       <c r="A30" t="n" s="22">
@@ -27516,6 +27545,7 @@
       <c r="M30"/>
       <c r="N30"/>
       <c r="O30"/>
+      <c r="P30"/>
     </row>
     <row r="31">
       <c r="A31" t="n" s="22">
@@ -27547,6 +27577,7 @@
       <c r="M31"/>
       <c r="N31"/>
       <c r="O31"/>
+      <c r="P31"/>
     </row>
     <row r="32">
       <c r="A32" t="n" s="22">
@@ -27578,6 +27609,7 @@
       <c r="M32"/>
       <c r="N32"/>
       <c r="O32"/>
+      <c r="P32"/>
     </row>
     <row r="33">
       <c r="A33" t="n" s="22">
@@ -27609,6 +27641,7 @@
       <c r="M33"/>
       <c r="N33"/>
       <c r="O33"/>
+      <c r="P33"/>
     </row>
     <row r="34">
       <c r="A34" t="n" s="22">
@@ -27640,6 +27673,7 @@
       <c r="M34"/>
       <c r="N34"/>
       <c r="O34"/>
+      <c r="P34"/>
     </row>
     <row r="35">
       <c r="A35" t="n" s="22">
@@ -27671,6 +27705,7 @@
       <c r="M35"/>
       <c r="N35"/>
       <c r="O35"/>
+      <c r="P35"/>
     </row>
     <row r="36">
       <c r="A36" t="n" s="22">
@@ -27702,6 +27737,7 @@
       <c r="M36"/>
       <c r="N36"/>
       <c r="O36"/>
+      <c r="P36"/>
     </row>
     <row r="37">
       <c r="A37" t="n" s="22">
@@ -27737,6 +27773,7 @@
       <c r="O37" t="s">
         <v>1242</v>
       </c>
+      <c r="P37"/>
     </row>
     <row r="38">
       <c r="A38" t="n" s="22">
@@ -27768,6 +27805,7 @@
       <c r="M38"/>
       <c r="N38"/>
       <c r="O38"/>
+      <c r="P38"/>
     </row>
     <row r="39">
       <c r="A39" t="n" s="22">
@@ -27799,6 +27837,7 @@
       <c r="M39"/>
       <c r="N39"/>
       <c r="O39"/>
+      <c r="P39"/>
     </row>
     <row r="40">
       <c r="A40" t="n" s="22">
@@ -27830,6 +27869,7 @@
       <c r="M40"/>
       <c r="N40"/>
       <c r="O40"/>
+      <c r="P40"/>
     </row>
     <row r="41">
       <c r="A41" t="n" s="22">
@@ -27863,6 +27903,7 @@
       <c r="M41"/>
       <c r="N41"/>
       <c r="O41"/>
+      <c r="P41"/>
     </row>
     <row r="42">
       <c r="A42" t="n" s="22">
@@ -27894,6 +27935,7 @@
       <c r="M42"/>
       <c r="N42"/>
       <c r="O42"/>
+      <c r="P42"/>
     </row>
     <row r="43">
       <c r="A43" t="n" s="22">
@@ -27925,6 +27967,7 @@
       <c r="M43"/>
       <c r="N43"/>
       <c r="O43"/>
+      <c r="P43"/>
     </row>
     <row r="44">
       <c r="A44" t="n" s="22">
@@ -27956,6 +27999,7 @@
       <c r="M44"/>
       <c r="N44"/>
       <c r="O44"/>
+      <c r="P44"/>
     </row>
     <row r="45">
       <c r="A45" t="n" s="22">
@@ -27987,6 +28031,7 @@
       <c r="M45"/>
       <c r="N45"/>
       <c r="O45"/>
+      <c r="P45"/>
     </row>
     <row r="46">
       <c r="A46" t="n" s="22">
@@ -28018,6 +28063,7 @@
       <c r="M46"/>
       <c r="N46"/>
       <c r="O46"/>
+      <c r="P46"/>
     </row>
     <row r="47">
       <c r="A47" t="n" s="22">
@@ -28049,6 +28095,7 @@
       <c r="M47"/>
       <c r="N47"/>
       <c r="O47"/>
+      <c r="P47"/>
     </row>
     <row r="48">
       <c r="A48" t="n" s="22">
@@ -28080,6 +28127,7 @@
       <c r="M48"/>
       <c r="N48"/>
       <c r="O48"/>
+      <c r="P48"/>
     </row>
     <row r="49">
       <c r="A49" t="n" s="22">
@@ -28111,6 +28159,7 @@
       <c r="M49"/>
       <c r="N49"/>
       <c r="O49"/>
+      <c r="P49"/>
     </row>
     <row r="50">
       <c r="A50" t="n" s="22">
@@ -28142,6 +28191,7 @@
       <c r="M50"/>
       <c r="N50"/>
       <c r="O50"/>
+      <c r="P50"/>
     </row>
     <row r="51">
       <c r="A51" t="n" s="22">
@@ -28173,6 +28223,7 @@
       <c r="M51"/>
       <c r="N51"/>
       <c r="O51"/>
+      <c r="P51"/>
     </row>
     <row r="52">
       <c r="A52" t="n" s="22">
@@ -28204,6 +28255,7 @@
       <c r="M52"/>
       <c r="N52"/>
       <c r="O52"/>
+      <c r="P52"/>
     </row>
     <row r="53">
       <c r="A53" t="n" s="22">
@@ -28235,6 +28287,7 @@
       <c r="M53"/>
       <c r="N53"/>
       <c r="O53"/>
+      <c r="P53"/>
     </row>
     <row r="54">
       <c r="A54" t="n" s="22">
@@ -28266,6 +28319,7 @@
       <c r="M54"/>
       <c r="N54"/>
       <c r="O54"/>
+      <c r="P54"/>
     </row>
     <row r="55">
       <c r="A55" t="n" s="22">
@@ -28299,6 +28353,7 @@
       <c r="M55"/>
       <c r="N55"/>
       <c r="O55"/>
+      <c r="P55"/>
     </row>
     <row r="56">
       <c r="A56" t="n" s="22">
@@ -28330,6 +28385,7 @@
       <c r="M56"/>
       <c r="N56"/>
       <c r="O56"/>
+      <c r="P56"/>
     </row>
     <row r="57">
       <c r="A57" t="n" s="22">
@@ -28361,6 +28417,7 @@
       <c r="M57"/>
       <c r="N57"/>
       <c r="O57"/>
+      <c r="P57"/>
     </row>
     <row r="58">
       <c r="A58" t="n" s="22">
@@ -28392,6 +28449,7 @@
       <c r="M58"/>
       <c r="N58"/>
       <c r="O58"/>
+      <c r="P58"/>
     </row>
     <row r="59">
       <c r="A59" t="n" s="22">
@@ -28425,6 +28483,7 @@
       <c r="M59"/>
       <c r="N59"/>
       <c r="O59"/>
+      <c r="P59"/>
     </row>
     <row r="60">
       <c r="A60" t="n" s="22">
@@ -28456,6 +28515,7 @@
       <c r="M60"/>
       <c r="N60"/>
       <c r="O60"/>
+      <c r="P60"/>
     </row>
     <row r="61">
       <c r="A61" t="n" s="22">
@@ -28487,6 +28547,7 @@
       <c r="M61"/>
       <c r="N61"/>
       <c r="O61"/>
+      <c r="P61"/>
     </row>
     <row r="62">
       <c r="A62" t="n" s="22">
@@ -28518,6 +28579,7 @@
       <c r="M62"/>
       <c r="N62"/>
       <c r="O62"/>
+      <c r="P62"/>
     </row>
     <row r="63">
       <c r="A63" t="n" s="22">
@@ -28551,6 +28613,7 @@
       <c r="M63"/>
       <c r="N63"/>
       <c r="O63"/>
+      <c r="P63"/>
     </row>
     <row r="64">
       <c r="A64" t="n" s="22">
@@ -28582,6 +28645,7 @@
       <c r="M64"/>
       <c r="N64"/>
       <c r="O64"/>
+      <c r="P64"/>
     </row>
     <row r="65">
       <c r="A65" t="n" s="22">
@@ -28613,6 +28677,7 @@
       <c r="M65"/>
       <c r="N65"/>
       <c r="O65"/>
+      <c r="P65"/>
     </row>
     <row r="66">
       <c r="A66" t="n" s="22">
@@ -28644,6 +28709,7 @@
       <c r="M66"/>
       <c r="N66"/>
       <c r="O66"/>
+      <c r="P66"/>
     </row>
     <row r="67">
       <c r="A67" t="n" s="22">
@@ -28677,6 +28743,7 @@
       <c r="M67"/>
       <c r="N67"/>
       <c r="O67"/>
+      <c r="P67"/>
     </row>
     <row r="68">
       <c r="A68" t="n" s="22">
@@ -28708,6 +28775,7 @@
       <c r="M68"/>
       <c r="N68"/>
       <c r="O68"/>
+      <c r="P68"/>
     </row>
     <row r="69">
       <c r="A69" t="n" s="22">
@@ -28741,6 +28809,7 @@
       <c r="M69"/>
       <c r="N69"/>
       <c r="O69"/>
+      <c r="P69"/>
     </row>
     <row r="70">
       <c r="A70" t="n" s="22">
@@ -28774,6 +28843,7 @@
       <c r="M70"/>
       <c r="N70"/>
       <c r="O70"/>
+      <c r="P70"/>
     </row>
     <row r="71">
       <c r="A71" t="n" s="22">
@@ -28805,6 +28875,7 @@
       <c r="M71"/>
       <c r="N71"/>
       <c r="O71"/>
+      <c r="P71"/>
     </row>
     <row r="72">
       <c r="A72" t="n" s="22">
@@ -28836,6 +28907,7 @@
       <c r="M72"/>
       <c r="N72"/>
       <c r="O72"/>
+      <c r="P72"/>
     </row>
     <row r="73">
       <c r="A73" t="n" s="22">
@@ -28867,6 +28939,7 @@
       <c r="M73"/>
       <c r="N73"/>
       <c r="O73"/>
+      <c r="P73"/>
     </row>
     <row r="74">
       <c r="A74" t="n" s="22">
@@ -28898,6 +28971,7 @@
       <c r="M74"/>
       <c r="N74"/>
       <c r="O74"/>
+      <c r="P74"/>
     </row>
     <row r="75">
       <c r="A75" t="n" s="22">
@@ -28929,6 +29003,7 @@
       <c r="M75"/>
       <c r="N75"/>
       <c r="O75"/>
+      <c r="P75"/>
     </row>
     <row r="76">
       <c r="A76" t="n" s="22">
@@ -28960,6 +29035,7 @@
       <c r="M76"/>
       <c r="N76"/>
       <c r="O76"/>
+      <c r="P76"/>
     </row>
     <row r="77">
       <c r="A77" t="n" s="22">
@@ -28991,6 +29067,7 @@
       <c r="M77"/>
       <c r="N77"/>
       <c r="O77"/>
+      <c r="P77"/>
     </row>
     <row r="78">
       <c r="A78" t="n" s="22">
@@ -29022,6 +29099,7 @@
       <c r="M78"/>
       <c r="N78"/>
       <c r="O78"/>
+      <c r="P78"/>
     </row>
     <row r="79">
       <c r="A79" t="n" s="22">
@@ -29053,6 +29131,7 @@
       <c r="M79"/>
       <c r="N79"/>
       <c r="O79"/>
+      <c r="P79"/>
     </row>
     <row r="80">
       <c r="A80" t="n" s="22">
@@ -29084,6 +29163,7 @@
       <c r="M80"/>
       <c r="N80"/>
       <c r="O80"/>
+      <c r="P80"/>
     </row>
     <row r="81">
       <c r="A81" t="n" s="22">
@@ -29115,6 +29195,7 @@
       <c r="M81"/>
       <c r="N81"/>
       <c r="O81"/>
+      <c r="P81"/>
     </row>
     <row r="82">
       <c r="A82" t="n" s="22">
@@ -29146,6 +29227,7 @@
       <c r="M82"/>
       <c r="N82"/>
       <c r="O82"/>
+      <c r="P82"/>
     </row>
     <row r="83">
       <c r="A83" t="n" s="22">
@@ -29177,6 +29259,7 @@
       <c r="M83"/>
       <c r="N83"/>
       <c r="O83"/>
+      <c r="P83"/>
     </row>
     <row r="84">
       <c r="A84" t="n" s="22">
@@ -29208,6 +29291,7 @@
       <c r="M84"/>
       <c r="N84"/>
       <c r="O84"/>
+      <c r="P84"/>
     </row>
     <row r="85">
       <c r="A85" t="n" s="22">
@@ -29237,6 +29321,7 @@
       <c r="M85"/>
       <c r="N85"/>
       <c r="O85"/>
+      <c r="P85"/>
     </row>
     <row r="86">
       <c r="A86" t="n" s="22">
@@ -29266,6 +29351,7 @@
       <c r="M86"/>
       <c r="N86"/>
       <c r="O86"/>
+      <c r="P86"/>
     </row>
     <row r="87">
       <c r="A87" t="n" s="22">
@@ -29295,6 +29381,7 @@
       <c r="M87"/>
       <c r="N87"/>
       <c r="O87"/>
+      <c r="P87"/>
     </row>
     <row r="88">
       <c r="A88" t="n" s="22">
@@ -29324,6 +29411,7 @@
       <c r="M88"/>
       <c r="N88"/>
       <c r="O88"/>
+      <c r="P88"/>
     </row>
     <row r="89">
       <c r="A89" t="n" s="22">
@@ -29353,6 +29441,7 @@
       <c r="M89"/>
       <c r="N89"/>
       <c r="O89"/>
+      <c r="P89"/>
     </row>
     <row r="90">
       <c r="A90" t="n" s="22">
@@ -29382,6 +29471,7 @@
       <c r="M90"/>
       <c r="N90"/>
       <c r="O90"/>
+      <c r="P90"/>
     </row>
     <row r="91">
       <c r="A91" t="n" s="22">
@@ -29413,6 +29503,7 @@
       <c r="M91"/>
       <c r="N91"/>
       <c r="O91"/>
+      <c r="P91"/>
     </row>
     <row r="92">
       <c r="A92" t="n" s="22">
@@ -29442,6 +29533,7 @@
       <c r="M92"/>
       <c r="N92"/>
       <c r="O92"/>
+      <c r="P92"/>
     </row>
     <row r="93">
       <c r="A93" t="n" s="22">
@@ -29473,6 +29565,7 @@
       <c r="M93"/>
       <c r="N93"/>
       <c r="O93"/>
+      <c r="P93"/>
     </row>
     <row r="94">
       <c r="A94" t="n" s="22">
@@ -29502,6 +29595,7 @@
       <c r="M94"/>
       <c r="N94"/>
       <c r="O94"/>
+      <c r="P94"/>
     </row>
     <row r="95">
       <c r="A95" t="n" s="22">
@@ -29533,6 +29627,7 @@
       <c r="M95"/>
       <c r="N95"/>
       <c r="O95"/>
+      <c r="P95"/>
     </row>
     <row r="96">
       <c r="A96" t="n" s="22">
@@ -29562,6 +29657,7 @@
       <c r="M96"/>
       <c r="N96"/>
       <c r="O96"/>
+      <c r="P96"/>
     </row>
     <row r="97">
       <c r="A97" t="n" s="22">
@@ -29591,6 +29687,7 @@
       <c r="M97"/>
       <c r="N97"/>
       <c r="O97"/>
+      <c r="P97"/>
     </row>
     <row r="98">
       <c r="A98" t="n" s="22">
@@ -29622,6 +29719,7 @@
       <c r="M98"/>
       <c r="N98"/>
       <c r="O98"/>
+      <c r="P98"/>
     </row>
     <row r="99">
       <c r="A99" t="n" s="22">
@@ -29651,6 +29749,7 @@
       <c r="M99"/>
       <c r="N99"/>
       <c r="O99"/>
+      <c r="P99"/>
     </row>
     <row r="100">
       <c r="A100" t="n" s="22">
@@ -29680,6 +29779,7 @@
       <c r="M100"/>
       <c r="N100"/>
       <c r="O100"/>
+      <c r="P100"/>
     </row>
     <row r="101">
       <c r="A101" t="n" s="22">
@@ -29711,6 +29811,7 @@
       <c r="M101"/>
       <c r="N101"/>
       <c r="O101"/>
+      <c r="P101"/>
     </row>
     <row r="102">
       <c r="A102" t="n" s="22">
@@ -29742,6 +29843,7 @@
       <c r="M102"/>
       <c r="N102"/>
       <c r="O102"/>
+      <c r="P102"/>
     </row>
     <row r="103">
       <c r="A103" t="n" s="22">
@@ -29773,6 +29875,7 @@
       <c r="M103"/>
       <c r="N103"/>
       <c r="O103"/>
+      <c r="P103"/>
     </row>
     <row r="104">
       <c r="A104" t="n" s="22">
@@ -29804,6 +29907,7 @@
       <c r="M104"/>
       <c r="N104"/>
       <c r="O104"/>
+      <c r="P104"/>
     </row>
     <row r="105">
       <c r="A105" t="n" s="22">
@@ -29835,6 +29939,7 @@
       <c r="M105"/>
       <c r="N105"/>
       <c r="O105"/>
+      <c r="P105"/>
     </row>
     <row r="106">
       <c r="A106" t="n" s="22">
@@ -29866,6 +29971,7 @@
       <c r="M106"/>
       <c r="N106"/>
       <c r="O106"/>
+      <c r="P106"/>
     </row>
     <row r="107">
       <c r="A107" t="n" s="22">
@@ -29897,6 +30003,7 @@
       <c r="M107"/>
       <c r="N107"/>
       <c r="O107"/>
+      <c r="P107"/>
     </row>
     <row r="108">
       <c r="A108" t="n" s="22">
@@ -29930,6 +30037,7 @@
       <c r="M108"/>
       <c r="N108"/>
       <c r="O108"/>
+      <c r="P108"/>
     </row>
     <row r="109">
       <c r="A109" t="n" s="22">
@@ -29963,6 +30071,7 @@
       <c r="M109"/>
       <c r="N109"/>
       <c r="O109"/>
+      <c r="P109"/>
     </row>
     <row r="110">
       <c r="A110" t="n" s="22">
@@ -29994,6 +30103,7 @@
       <c r="M110"/>
       <c r="N110"/>
       <c r="O110"/>
+      <c r="P110"/>
     </row>
     <row r="111">
       <c r="A111" t="n" s="22">
@@ -30025,6 +30135,7 @@
       <c r="M111"/>
       <c r="N111"/>
       <c r="O111"/>
+      <c r="P111"/>
     </row>
     <row r="112">
       <c r="A112" t="n" s="22">
@@ -30056,6 +30167,7 @@
       <c r="M112"/>
       <c r="N112"/>
       <c r="O112"/>
+      <c r="P112"/>
     </row>
     <row r="113">
       <c r="A113" t="n" s="22">
@@ -30089,6 +30201,7 @@
       <c r="M113"/>
       <c r="N113"/>
       <c r="O113"/>
+      <c r="P113"/>
     </row>
     <row r="114">
       <c r="A114" t="n" s="22">
@@ -30122,6 +30235,7 @@
       <c r="M114"/>
       <c r="N114"/>
       <c r="O114"/>
+      <c r="P114"/>
     </row>
     <row r="115">
       <c r="A115" t="n" s="22">
@@ -30153,6 +30267,7 @@
       <c r="M115"/>
       <c r="N115"/>
       <c r="O115"/>
+      <c r="P115"/>
     </row>
     <row r="116">
       <c r="A116" t="n" s="22">
@@ -30184,6 +30299,7 @@
       <c r="M116"/>
       <c r="N116"/>
       <c r="O116"/>
+      <c r="P116"/>
     </row>
     <row r="117">
       <c r="A117" t="n" s="22">
@@ -30215,6 +30331,7 @@
       <c r="M117"/>
       <c r="N117"/>
       <c r="O117"/>
+      <c r="P117"/>
     </row>
     <row r="118">
       <c r="A118" t="n" s="22">
@@ -30248,6 +30365,7 @@
       <c r="M118"/>
       <c r="N118"/>
       <c r="O118"/>
+      <c r="P118"/>
     </row>
     <row r="119">
       <c r="A119" t="n" s="22">
@@ -30281,6 +30399,7 @@
       <c r="M119"/>
       <c r="N119"/>
       <c r="O119"/>
+      <c r="P119"/>
     </row>
     <row r="120">
       <c r="A120" t="n" s="22">
@@ -30312,6 +30431,7 @@
       <c r="M120"/>
       <c r="N120"/>
       <c r="O120"/>
+      <c r="P120"/>
     </row>
     <row r="121">
       <c r="A121" t="n" s="22">
@@ -30343,6 +30463,7 @@
       <c r="M121"/>
       <c r="N121"/>
       <c r="O121"/>
+      <c r="P121"/>
     </row>
     <row r="122">
       <c r="A122" t="n" s="22">
@@ -30374,6 +30495,7 @@
       <c r="M122"/>
       <c r="N122"/>
       <c r="O122"/>
+      <c r="P122"/>
     </row>
     <row r="123">
       <c r="A123" t="n" s="22">
@@ -30407,6 +30529,7 @@
       <c r="M123"/>
       <c r="N123"/>
       <c r="O123"/>
+      <c r="P123"/>
     </row>
     <row r="124">
       <c r="A124" t="n" s="22">
@@ -30440,6 +30563,7 @@
       <c r="M124"/>
       <c r="N124"/>
       <c r="O124"/>
+      <c r="P124"/>
     </row>
     <row r="125">
       <c r="A125" t="n" s="22">
@@ -30471,6 +30595,7 @@
       <c r="M125"/>
       <c r="N125"/>
       <c r="O125"/>
+      <c r="P125"/>
     </row>
     <row r="126">
       <c r="A126" t="n" s="22">
@@ -30502,6 +30627,7 @@
       <c r="M126"/>
       <c r="N126"/>
       <c r="O126"/>
+      <c r="P126"/>
     </row>
     <row r="127">
       <c r="A127" t="n" s="22">
@@ -30533,6 +30659,7 @@
       <c r="M127"/>
       <c r="N127"/>
       <c r="O127"/>
+      <c r="P127"/>
     </row>
     <row r="128">
       <c r="A128" t="n" s="22">
@@ -30566,6 +30693,7 @@
       <c r="M128"/>
       <c r="N128"/>
       <c r="O128"/>
+      <c r="P128"/>
     </row>
     <row r="129">
       <c r="A129" t="n" s="22">
@@ -30599,6 +30727,7 @@
       <c r="M129"/>
       <c r="N129"/>
       <c r="O129"/>
+      <c r="P129"/>
     </row>
     <row r="130">
       <c r="A130" t="n" s="22">
@@ -30630,6 +30759,7 @@
       <c r="M130"/>
       <c r="N130"/>
       <c r="O130"/>
+      <c r="P130"/>
     </row>
     <row r="131">
       <c r="A131" t="n" s="22">
@@ -30661,6 +30791,7 @@
       <c r="M131"/>
       <c r="N131"/>
       <c r="O131"/>
+      <c r="P131"/>
     </row>
     <row r="132">
       <c r="A132" t="n" s="22">
@@ -30694,6 +30825,7 @@
       <c r="M132"/>
       <c r="N132"/>
       <c r="O132"/>
+      <c r="P132"/>
     </row>
     <row r="133">
       <c r="A133" t="n" s="22">
@@ -30727,6 +30859,7 @@
       <c r="M133"/>
       <c r="N133"/>
       <c r="O133"/>
+      <c r="P133"/>
     </row>
     <row r="134">
       <c r="A134" t="n" s="22">
@@ -30758,6 +30891,7 @@
       <c r="M134"/>
       <c r="N134"/>
       <c r="O134"/>
+      <c r="P134"/>
     </row>
     <row r="135">
       <c r="A135" t="n" s="22">
@@ -30789,6 +30923,7 @@
       <c r="M135"/>
       <c r="N135"/>
       <c r="O135"/>
+      <c r="P135"/>
     </row>
     <row r="136">
       <c r="A136" t="n" s="22">
@@ -30822,6 +30957,7 @@
       <c r="M136"/>
       <c r="N136"/>
       <c r="O136"/>
+      <c r="P136"/>
     </row>
     <row r="137">
       <c r="A137" t="n" s="22">
@@ -30855,6 +30991,7 @@
       <c r="M137"/>
       <c r="N137"/>
       <c r="O137"/>
+      <c r="P137"/>
     </row>
     <row r="138">
       <c r="A138" t="n" s="22">
@@ -30886,6 +31023,7 @@
       <c r="M138"/>
       <c r="N138"/>
       <c r="O138"/>
+      <c r="P138"/>
     </row>
     <row r="139">
       <c r="A139" t="n" s="22">
@@ -30917,6 +31055,7 @@
       <c r="M139"/>
       <c r="N139"/>
       <c r="O139"/>
+      <c r="P139"/>
     </row>
     <row r="140">
       <c r="A140" t="n" s="22">
@@ -30950,6 +31089,7 @@
       <c r="M140"/>
       <c r="N140"/>
       <c r="O140"/>
+      <c r="P140"/>
     </row>
     <row r="141">
       <c r="A141" t="n" s="22">
@@ -30983,6 +31123,7 @@
       <c r="M141"/>
       <c r="N141"/>
       <c r="O141"/>
+      <c r="P141"/>
     </row>
     <row r="142">
       <c r="A142" t="n" s="22">
@@ -31014,6 +31155,7 @@
       <c r="M142"/>
       <c r="N142"/>
       <c r="O142"/>
+      <c r="P142"/>
     </row>
     <row r="143">
       <c r="A143" t="n" s="22">
@@ -31045,6 +31187,7 @@
       <c r="M143"/>
       <c r="N143"/>
       <c r="O143"/>
+      <c r="P143"/>
     </row>
     <row r="144">
       <c r="A144" t="n" s="22">
@@ -31076,6 +31219,7 @@
       <c r="M144"/>
       <c r="N144"/>
       <c r="O144"/>
+      <c r="P144"/>
     </row>
     <row r="145">
       <c r="A145" t="n" s="22">
@@ -31107,6 +31251,7 @@
       <c r="M145"/>
       <c r="N145"/>
       <c r="O145"/>
+      <c r="P145"/>
     </row>
     <row r="146">
       <c r="A146" t="n" s="22">
@@ -31138,6 +31283,7 @@
       <c r="M146"/>
       <c r="N146"/>
       <c r="O146"/>
+      <c r="P146"/>
     </row>
     <row r="147">
       <c r="A147" t="n" s="22">
@@ -31169,6 +31315,7 @@
       <c r="M147"/>
       <c r="N147"/>
       <c r="O147"/>
+      <c r="P147"/>
     </row>
     <row r="148">
       <c r="A148" t="n" s="22">
@@ -31200,6 +31347,7 @@
       <c r="M148"/>
       <c r="N148"/>
       <c r="O148"/>
+      <c r="P148"/>
     </row>
     <row r="149">
       <c r="A149" t="n" s="22">
@@ -31231,6 +31379,7 @@
       <c r="M149"/>
       <c r="N149"/>
       <c r="O149"/>
+      <c r="P149"/>
     </row>
     <row r="150">
       <c r="A150" t="n" s="22">
@@ -31262,6 +31411,7 @@
       <c r="M150"/>
       <c r="N150"/>
       <c r="O150"/>
+      <c r="P150"/>
     </row>
     <row r="151">
       <c r="A151" t="n" s="22">
@@ -31295,6 +31445,7 @@
       <c r="M151"/>
       <c r="N151"/>
       <c r="O151"/>
+      <c r="P151"/>
     </row>
     <row r="152">
       <c r="A152" t="n" s="22">
@@ -31328,6 +31479,7 @@
       <c r="M152"/>
       <c r="N152"/>
       <c r="O152"/>
+      <c r="P152"/>
     </row>
     <row r="153">
       <c r="A153" t="n" s="22">
@@ -31361,6 +31513,7 @@
       <c r="M153"/>
       <c r="N153"/>
       <c r="O153"/>
+      <c r="P153"/>
     </row>
     <row r="154">
       <c r="A154" t="n" s="22">
@@ -31392,6 +31545,7 @@
       <c r="M154"/>
       <c r="N154"/>
       <c r="O154"/>
+      <c r="P154"/>
     </row>
     <row r="155">
       <c r="A155" t="n" s="22">
@@ -31423,6 +31577,7 @@
       <c r="M155"/>
       <c r="N155"/>
       <c r="O155"/>
+      <c r="P155"/>
     </row>
     <row r="156">
       <c r="A156" t="n" s="22">
@@ -31454,6 +31609,7 @@
       <c r="M156"/>
       <c r="N156"/>
       <c r="O156"/>
+      <c r="P156"/>
     </row>
     <row r="157">
       <c r="A157" t="n" s="22">
@@ -31487,6 +31643,7 @@
       <c r="M157"/>
       <c r="N157"/>
       <c r="O157"/>
+      <c r="P157"/>
     </row>
     <row r="158">
       <c r="A158" t="n" s="22">
@@ -31520,6 +31677,7 @@
       <c r="M158"/>
       <c r="N158"/>
       <c r="O158"/>
+      <c r="P158"/>
     </row>
     <row r="159">
       <c r="A159" t="n" s="22">
@@ -31551,6 +31709,7 @@
       <c r="M159"/>
       <c r="N159"/>
       <c r="O159"/>
+      <c r="P159"/>
     </row>
     <row r="160">
       <c r="A160" t="n" s="22">
@@ -31582,6 +31741,7 @@
       <c r="M160"/>
       <c r="N160"/>
       <c r="O160"/>
+      <c r="P160"/>
     </row>
     <row r="161">
       <c r="A161" t="n" s="22">
@@ -31613,6 +31773,7 @@
       <c r="M161"/>
       <c r="N161"/>
       <c r="O161"/>
+      <c r="P161"/>
     </row>
     <row r="162">
       <c r="A162" t="n" s="22">
@@ -31646,6 +31807,7 @@
       <c r="M162"/>
       <c r="N162"/>
       <c r="O162"/>
+      <c r="P162"/>
     </row>
     <row r="163">
       <c r="A163" t="n" s="22">
@@ -31679,6 +31841,7 @@
       <c r="M163"/>
       <c r="N163"/>
       <c r="O163"/>
+      <c r="P163"/>
     </row>
     <row r="164">
       <c r="A164" t="n" s="22">
@@ -31710,6 +31873,7 @@
       <c r="M164"/>
       <c r="N164"/>
       <c r="O164"/>
+      <c r="P164"/>
     </row>
     <row r="165">
       <c r="A165" t="n" s="22">
@@ -31741,6 +31905,7 @@
       <c r="M165"/>
       <c r="N165"/>
       <c r="O165"/>
+      <c r="P165"/>
     </row>
     <row r="166">
       <c r="A166" t="n" s="22">
@@ -31772,6 +31937,7 @@
       <c r="M166"/>
       <c r="N166"/>
       <c r="O166"/>
+      <c r="P166"/>
     </row>
     <row r="167">
       <c r="A167" t="n" s="22">
@@ -31803,6 +31969,7 @@
       <c r="M167"/>
       <c r="N167"/>
       <c r="O167"/>
+      <c r="P167"/>
     </row>
     <row r="168">
       <c r="A168" t="n" s="22">
@@ -31834,6 +32001,7 @@
       <c r="M168"/>
       <c r="N168"/>
       <c r="O168"/>
+      <c r="P168"/>
     </row>
     <row r="169">
       <c r="A169" t="n" s="22">
@@ -31865,6 +32033,7 @@
       <c r="M169"/>
       <c r="N169"/>
       <c r="O169"/>
+      <c r="P169"/>
     </row>
     <row r="170">
       <c r="A170" t="n" s="22">
@@ -31896,6 +32065,7 @@
       <c r="M170"/>
       <c r="N170"/>
       <c r="O170"/>
+      <c r="P170"/>
     </row>
     <row r="171">
       <c r="A171" t="n" s="22">
@@ -31927,6 +32097,7 @@
       <c r="M171"/>
       <c r="N171"/>
       <c r="O171"/>
+      <c r="P171"/>
     </row>
     <row r="172">
       <c r="A172" t="n" s="22">
@@ -31958,6 +32129,7 @@
       <c r="M172"/>
       <c r="N172"/>
       <c r="O172"/>
+      <c r="P172"/>
     </row>
     <row r="173">
       <c r="A173" t="n" s="22">
@@ -31989,6 +32161,7 @@
       <c r="M173"/>
       <c r="N173"/>
       <c r="O173"/>
+      <c r="P173"/>
     </row>
     <row r="174">
       <c r="A174" t="n" s="22">
@@ -32022,6 +32195,7 @@
       <c r="M174"/>
       <c r="N174"/>
       <c r="O174"/>
+      <c r="P174"/>
     </row>
     <row r="175">
       <c r="A175" t="n" s="22">
@@ -32055,6 +32229,7 @@
       <c r="M175"/>
       <c r="N175"/>
       <c r="O175"/>
+      <c r="P175"/>
     </row>
     <row r="176">
       <c r="A176" t="n" s="22">
@@ -32086,6 +32261,7 @@
       <c r="M176"/>
       <c r="N176"/>
       <c r="O176"/>
+      <c r="P176"/>
     </row>
     <row r="177">
       <c r="A177" t="n" s="22">
@@ -32117,6 +32293,7 @@
       <c r="M177"/>
       <c r="N177"/>
       <c r="O177"/>
+      <c r="P177"/>
     </row>
     <row r="178">
       <c r="A178" t="n" s="22">
@@ -32148,6 +32325,7 @@
       <c r="M178"/>
       <c r="N178"/>
       <c r="O178"/>
+      <c r="P178"/>
     </row>
     <row r="179">
       <c r="A179" t="n" s="22">
@@ -32181,6 +32359,7 @@
       <c r="M179"/>
       <c r="N179"/>
       <c r="O179"/>
+      <c r="P179"/>
     </row>
     <row r="180">
       <c r="A180" t="n" s="22">
@@ -32214,6 +32393,7 @@
       <c r="M180"/>
       <c r="N180"/>
       <c r="O180"/>
+      <c r="P180"/>
     </row>
     <row r="181">
       <c r="A181" t="n" s="22">
@@ -32245,6 +32425,7 @@
       <c r="M181"/>
       <c r="N181"/>
       <c r="O181"/>
+      <c r="P181"/>
     </row>
     <row r="182">
       <c r="A182" t="n" s="22">
@@ -32276,6 +32457,7 @@
       <c r="M182"/>
       <c r="N182"/>
       <c r="O182"/>
+      <c r="P182"/>
     </row>
     <row r="183">
       <c r="A183" t="n" s="22">
@@ -32307,6 +32489,7 @@
       <c r="M183"/>
       <c r="N183"/>
       <c r="O183"/>
+      <c r="P183"/>
     </row>
     <row r="184">
       <c r="A184" t="n" s="22">
@@ -32340,6 +32523,7 @@
       <c r="M184"/>
       <c r="N184"/>
       <c r="O184"/>
+      <c r="P184"/>
     </row>
     <row r="185">
       <c r="A185" t="n" s="22">
@@ -32373,6 +32557,7 @@
       <c r="M185"/>
       <c r="N185"/>
       <c r="O185"/>
+      <c r="P185"/>
     </row>
     <row r="186">
       <c r="A186" t="n" s="22">
@@ -32404,6 +32589,7 @@
       <c r="M186"/>
       <c r="N186"/>
       <c r="O186"/>
+      <c r="P186"/>
     </row>
     <row r="187">
       <c r="A187" t="n" s="22">
@@ -32435,6 +32621,7 @@
       <c r="M187"/>
       <c r="N187"/>
       <c r="O187"/>
+      <c r="P187"/>
     </row>
     <row r="188">
       <c r="A188" t="n" s="22">
@@ -32466,6 +32653,7 @@
       <c r="M188"/>
       <c r="N188"/>
       <c r="O188"/>
+      <c r="P188"/>
     </row>
     <row r="189">
       <c r="A189" t="n" s="22">
@@ -32497,6 +32685,7 @@
       <c r="M189"/>
       <c r="N189"/>
       <c r="O189"/>
+      <c r="P189"/>
     </row>
     <row r="190">
       <c r="A190" t="n" s="22">
@@ -32528,6 +32717,7 @@
       <c r="M190"/>
       <c r="N190"/>
       <c r="O190"/>
+      <c r="P190"/>
     </row>
     <row r="191">
       <c r="A191" t="n" s="22">
@@ -32559,6 +32749,7 @@
       <c r="M191"/>
       <c r="N191"/>
       <c r="O191"/>
+      <c r="P191"/>
     </row>
     <row r="192">
       <c r="A192" t="n" s="22">
@@ -32590,6 +32781,7 @@
       <c r="M192"/>
       <c r="N192"/>
       <c r="O192"/>
+      <c r="P192"/>
     </row>
     <row r="193">
       <c r="A193" t="n" s="22">
@@ -32621,6 +32813,7 @@
       <c r="M193"/>
       <c r="N193"/>
       <c r="O193"/>
+      <c r="P193"/>
     </row>
     <row r="194">
       <c r="A194" t="n" s="22">
@@ -32652,6 +32845,7 @@
       <c r="M194"/>
       <c r="N194"/>
       <c r="O194"/>
+      <c r="P194"/>
     </row>
     <row r="195">
       <c r="A195" t="n" s="22">
@@ -32685,6 +32879,7 @@
       <c r="M195"/>
       <c r="N195"/>
       <c r="O195"/>
+      <c r="P195"/>
     </row>
     <row r="196">
       <c r="A196" t="n" s="22">
@@ -32718,6 +32913,7 @@
       <c r="M196"/>
       <c r="N196"/>
       <c r="O196"/>
+      <c r="P196"/>
     </row>
     <row r="197">
       <c r="A197" t="n" s="22">
@@ -32751,6 +32947,7 @@
       <c r="M197"/>
       <c r="N197"/>
       <c r="O197"/>
+      <c r="P197"/>
     </row>
     <row r="198">
       <c r="A198" t="n" s="22">
@@ -32782,6 +32979,7 @@
       <c r="M198"/>
       <c r="N198"/>
       <c r="O198"/>
+      <c r="P198"/>
     </row>
     <row r="199">
       <c r="A199" t="n" s="22">
@@ -32813,6 +33011,7 @@
       <c r="M199"/>
       <c r="N199"/>
       <c r="O199"/>
+      <c r="P199"/>
     </row>
     <row r="200">
       <c r="A200" t="n" s="22">
@@ -32844,6 +33043,7 @@
       <c r="M200"/>
       <c r="N200"/>
       <c r="O200"/>
+      <c r="P200"/>
     </row>
     <row r="201">
       <c r="A201" t="n" s="22">
@@ -32877,6 +33077,7 @@
       <c r="M201"/>
       <c r="N201"/>
       <c r="O201"/>
+      <c r="P201"/>
     </row>
     <row r="202">
       <c r="A202" t="n" s="22">
@@ -32910,6 +33111,7 @@
       <c r="M202"/>
       <c r="N202"/>
       <c r="O202"/>
+      <c r="P202"/>
     </row>
     <row r="203">
       <c r="A203" t="n" s="22">
@@ -32941,6 +33143,7 @@
       <c r="M203"/>
       <c r="N203"/>
       <c r="O203"/>
+      <c r="P203"/>
     </row>
     <row r="204">
       <c r="A204" t="n" s="22">
@@ -32972,6 +33175,7 @@
       <c r="M204"/>
       <c r="N204"/>
       <c r="O204"/>
+      <c r="P204"/>
     </row>
     <row r="205">
       <c r="A205" t="n" s="22">
@@ -33003,6 +33207,7 @@
       <c r="M205"/>
       <c r="N205"/>
       <c r="O205"/>
+      <c r="P205"/>
     </row>
     <row r="206">
       <c r="A206" t="n" s="22">
@@ -33036,6 +33241,7 @@
       <c r="M206"/>
       <c r="N206"/>
       <c r="O206"/>
+      <c r="P206"/>
     </row>
     <row r="207">
       <c r="A207" t="n" s="22">
@@ -33069,6 +33275,7 @@
       <c r="M207"/>
       <c r="N207"/>
       <c r="O207"/>
+      <c r="P207"/>
     </row>
     <row r="208">
       <c r="A208" t="n" s="22">
@@ -33100,6 +33307,7 @@
       <c r="M208"/>
       <c r="N208"/>
       <c r="O208"/>
+      <c r="P208"/>
     </row>
     <row r="209">
       <c r="A209" t="n" s="22">
@@ -33131,6 +33339,7 @@
       <c r="M209"/>
       <c r="N209"/>
       <c r="O209"/>
+      <c r="P209"/>
     </row>
     <row r="210">
       <c r="A210" t="n" s="22">
@@ -33162,6 +33371,7 @@
       <c r="M210"/>
       <c r="N210"/>
       <c r="O210"/>
+      <c r="P210"/>
     </row>
     <row r="211">
       <c r="A211" t="n" s="22">
@@ -33193,6 +33403,7 @@
       <c r="M211"/>
       <c r="N211"/>
       <c r="O211"/>
+      <c r="P211"/>
     </row>
     <row r="212">
       <c r="A212" t="n" s="22">
@@ -33224,6 +33435,7 @@
       <c r="M212"/>
       <c r="N212"/>
       <c r="O212"/>
+      <c r="P212"/>
     </row>
     <row r="213">
       <c r="A213" t="n" s="22">
@@ -33255,6 +33467,7 @@
       <c r="M213"/>
       <c r="N213"/>
       <c r="O213"/>
+      <c r="P213"/>
     </row>
     <row r="214">
       <c r="A214" t="n" s="22">
@@ -33286,6 +33499,7 @@
       <c r="M214"/>
       <c r="N214"/>
       <c r="O214"/>
+      <c r="P214"/>
     </row>
     <row r="215">
       <c r="A215" t="n" s="22">
@@ -33317,6 +33531,7 @@
       <c r="M215"/>
       <c r="N215"/>
       <c r="O215"/>
+      <c r="P215"/>
     </row>
     <row r="216">
       <c r="A216" t="n" s="22">
@@ -33348,6 +33563,7 @@
       <c r="M216"/>
       <c r="N216"/>
       <c r="O216"/>
+      <c r="P216"/>
     </row>
     <row r="217">
       <c r="A217" t="n" s="22">
@@ -33379,6 +33595,7 @@
       <c r="M217"/>
       <c r="N217"/>
       <c r="O217"/>
+      <c r="P217"/>
     </row>
     <row r="218">
       <c r="A218" t="n" s="22">
@@ -33412,6 +33629,7 @@
       <c r="M218"/>
       <c r="N218"/>
       <c r="O218"/>
+      <c r="P218"/>
     </row>
     <row r="219">
       <c r="A219" t="n" s="22">
@@ -33445,6 +33663,7 @@
       <c r="M219"/>
       <c r="N219"/>
       <c r="O219"/>
+      <c r="P219"/>
     </row>
     <row r="220">
       <c r="A220" t="n" s="22">
@@ -33476,6 +33695,7 @@
       <c r="M220"/>
       <c r="N220"/>
       <c r="O220"/>
+      <c r="P220"/>
     </row>
     <row r="221">
       <c r="A221" t="n" s="22">
@@ -33507,6 +33727,7 @@
       <c r="M221"/>
       <c r="N221"/>
       <c r="O221"/>
+      <c r="P221"/>
     </row>
     <row r="222">
       <c r="A222" t="n" s="22">
@@ -33538,6 +33759,7 @@
       <c r="M222"/>
       <c r="N222"/>
       <c r="O222"/>
+      <c r="P222"/>
     </row>
     <row r="223">
       <c r="A223" t="n" s="22">
@@ -33571,6 +33793,7 @@
       <c r="M223"/>
       <c r="N223"/>
       <c r="O223"/>
+      <c r="P223"/>
     </row>
     <row r="224">
       <c r="A224" t="n" s="22">
@@ -33604,6 +33827,7 @@
       <c r="M224"/>
       <c r="N224"/>
       <c r="O224"/>
+      <c r="P224"/>
     </row>
     <row r="225">
       <c r="A225" t="n" s="22">
@@ -33635,6 +33859,7 @@
       <c r="M225"/>
       <c r="N225"/>
       <c r="O225"/>
+      <c r="P225"/>
     </row>
     <row r="226">
       <c r="A226" t="n" s="22">
@@ -33666,6 +33891,7 @@
       <c r="M226"/>
       <c r="N226"/>
       <c r="O226"/>
+      <c r="P226"/>
     </row>
     <row r="227">
       <c r="A227" t="n" s="22">
@@ -33697,6 +33923,7 @@
       <c r="M227"/>
       <c r="N227"/>
       <c r="O227"/>
+      <c r="P227"/>
     </row>
     <row r="228">
       <c r="A228" t="n" s="22">
@@ -33730,6 +33957,7 @@
       <c r="M228"/>
       <c r="N228"/>
       <c r="O228"/>
+      <c r="P228"/>
     </row>
     <row r="229">
       <c r="A229" t="n" s="22">
@@ -33763,6 +33991,7 @@
       <c r="M229"/>
       <c r="N229"/>
       <c r="O229"/>
+      <c r="P229"/>
     </row>
     <row r="230">
       <c r="A230" t="n" s="22">
@@ -33794,6 +34023,7 @@
       <c r="M230"/>
       <c r="N230"/>
       <c r="O230"/>
+      <c r="P230"/>
     </row>
     <row r="231">
       <c r="A231" t="n" s="22">
@@ -33825,6 +34055,7 @@
       <c r="M231"/>
       <c r="N231"/>
       <c r="O231"/>
+      <c r="P231"/>
     </row>
     <row r="232">
       <c r="A232" t="n" s="22">
@@ -33856,6 +34087,7 @@
       <c r="M232"/>
       <c r="N232"/>
       <c r="O232"/>
+      <c r="P232"/>
     </row>
     <row r="233">
       <c r="A233" t="n" s="22">
@@ -33887,6 +34119,7 @@
       <c r="M233"/>
       <c r="N233"/>
       <c r="O233"/>
+      <c r="P233"/>
     </row>
     <row r="234">
       <c r="A234" t="n" s="22">
@@ -33918,6 +34151,7 @@
       <c r="M234"/>
       <c r="N234"/>
       <c r="O234"/>
+      <c r="P234"/>
     </row>
     <row r="235">
       <c r="A235" t="n" s="22">
@@ -33949,6 +34183,7 @@
       <c r="M235"/>
       <c r="N235"/>
       <c r="O235"/>
+      <c r="P235"/>
     </row>
     <row r="236">
       <c r="A236" t="n" s="22">
@@ -33980,6 +34215,7 @@
       <c r="M236"/>
       <c r="N236"/>
       <c r="O236"/>
+      <c r="P236"/>
     </row>
     <row r="237">
       <c r="A237" t="n" s="22">
@@ -34011,6 +34247,7 @@
       <c r="M237"/>
       <c r="N237"/>
       <c r="O237"/>
+      <c r="P237"/>
     </row>
     <row r="238">
       <c r="A238" t="n" s="22">
@@ -34042,6 +34279,7 @@
       <c r="M238"/>
       <c r="N238"/>
       <c r="O238"/>
+      <c r="P238"/>
     </row>
     <row r="239">
       <c r="A239" t="n" s="22">
@@ -34073,6 +34311,7 @@
       <c r="M239"/>
       <c r="N239"/>
       <c r="O239"/>
+      <c r="P239"/>
     </row>
     <row r="240">
       <c r="A240" t="n" s="22">
@@ -34106,6 +34345,7 @@
       </c>
       <c r="N240"/>
       <c r="O240"/>
+      <c r="P240"/>
     </row>
     <row r="241">
       <c r="A241" t="n" s="22">
@@ -34137,6 +34377,7 @@
       <c r="M241"/>
       <c r="N241"/>
       <c r="O241"/>
+      <c r="P241"/>
     </row>
     <row r="242">
       <c r="A242" t="n" s="22">
@@ -34170,6 +34411,7 @@
       </c>
       <c r="N242"/>
       <c r="O242"/>
+      <c r="P242"/>
     </row>
     <row r="243">
       <c r="A243" t="n" s="22">
@@ -34203,6 +34445,7 @@
       <c r="M243"/>
       <c r="N243"/>
       <c r="O243"/>
+      <c r="P243"/>
     </row>
     <row r="244">
       <c r="A244" t="n" s="22">
@@ -34238,6 +34481,7 @@
       <c r="M244"/>
       <c r="N244"/>
       <c r="O244"/>
+      <c r="P244"/>
     </row>
     <row r="245">
       <c r="A245" t="n" s="22">
@@ -34269,6 +34513,7 @@
       <c r="M245"/>
       <c r="N245"/>
       <c r="O245"/>
+      <c r="P245"/>
     </row>
     <row r="246">
       <c r="A246" t="n" s="22">
@@ -34300,6 +34545,7 @@
       <c r="M246"/>
       <c r="N246"/>
       <c r="O246"/>
+      <c r="P246"/>
     </row>
     <row r="247">
       <c r="A247" t="n" s="22">
@@ -34331,6 +34577,7 @@
       <c r="M247"/>
       <c r="N247"/>
       <c r="O247"/>
+      <c r="P247"/>
     </row>
     <row r="248">
       <c r="A248" t="n" s="22">
@@ -34364,6 +34611,7 @@
       <c r="M248"/>
       <c r="N248"/>
       <c r="O248"/>
+      <c r="P248"/>
     </row>
     <row r="249">
       <c r="A249" t="n" s="22">
@@ -34395,6 +34643,7 @@
       <c r="M249"/>
       <c r="N249"/>
       <c r="O249"/>
+      <c r="P249"/>
     </row>
     <row r="250">
       <c r="A250" t="n" s="22">
@@ -34426,6 +34675,7 @@
       <c r="M250"/>
       <c r="N250"/>
       <c r="O250"/>
+      <c r="P250"/>
     </row>
     <row r="251">
       <c r="A251" t="n" s="22">
@@ -34457,6 +34707,7 @@
       <c r="M251"/>
       <c r="N251"/>
       <c r="O251"/>
+      <c r="P251"/>
     </row>
     <row r="252">
       <c r="A252" t="n" s="22">
@@ -34488,6 +34739,7 @@
       <c r="M252"/>
       <c r="N252"/>
       <c r="O252"/>
+      <c r="P252"/>
     </row>
     <row r="253">
       <c r="A253" t="n" s="22">
@@ -34519,6 +34771,7 @@
       <c r="M253"/>
       <c r="N253"/>
       <c r="O253"/>
+      <c r="P253"/>
     </row>
     <row r="254">
       <c r="A254" t="n" s="22">
@@ -34548,6 +34801,7 @@
       <c r="M254"/>
       <c r="N254"/>
       <c r="O254"/>
+      <c r="P254"/>
     </row>
     <row r="255">
       <c r="A255" t="n" s="22">
@@ -34577,6 +34831,7 @@
       <c r="M255"/>
       <c r="N255"/>
       <c r="O255"/>
+      <c r="P255"/>
     </row>
     <row r="256">
       <c r="A256" t="n" s="22">
@@ -34606,6 +34861,7 @@
       <c r="M256"/>
       <c r="N256"/>
       <c r="O256"/>
+      <c r="P256"/>
     </row>
     <row r="257">
       <c r="A257" t="n" s="22">
@@ -34613,16 +34869,16 @@
       </c>
       <c r="B257"/>
       <c r="C257" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="D257" t="s">
-        <v>774</v>
+        <v>768</v>
       </c>
       <c r="E257" t="s">
-        <v>313</v>
+        <v>443</v>
       </c>
       <c r="F257" t="s">
-        <v>666</v>
+        <v>658</v>
       </c>
       <c r="G257"/>
       <c r="H257"/>
@@ -34631,12 +34887,15 @@
         <v>1.0</v>
       </c>
       <c r="K257" t="s">
-        <v>1258</v>
+        <v>1227</v>
       </c>
       <c r="L257"/>
       <c r="M257"/>
       <c r="N257"/>
       <c r="O257"/>
+      <c r="P257" t="s">
+        <v>660</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="n" s="22">
@@ -34653,21 +34912,22 @@
         <v>313</v>
       </c>
       <c r="F258" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="G258"/>
       <c r="H258"/>
       <c r="I258"/>
       <c r="J258" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K258" t="s">
-        <v>1227</v>
+        <v>1258</v>
       </c>
       <c r="L258"/>
       <c r="M258"/>
       <c r="N258"/>
       <c r="O258"/>
+      <c r="P258"/>
     </row>
     <row r="259">
       <c r="A259" t="n" s="22">
@@ -34684,13 +34944,13 @@
         <v>313</v>
       </c>
       <c r="F259" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G259"/>
       <c r="H259"/>
       <c r="I259"/>
       <c r="J259" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K259" t="s">
         <v>1227</v>
@@ -34699,6 +34959,7 @@
       <c r="M259"/>
       <c r="N259"/>
       <c r="O259"/>
+      <c r="P259"/>
     </row>
     <row r="260">
       <c r="A260" t="n" s="22">
@@ -34709,19 +34970,19 @@
         <v>80</v>
       </c>
       <c r="D260" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="E260" t="s">
         <v>313</v>
       </c>
       <c r="F260" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="G260"/>
       <c r="H260"/>
       <c r="I260"/>
       <c r="J260" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K260" t="s">
         <v>1227</v>
@@ -34730,6 +34991,7 @@
       <c r="M260"/>
       <c r="N260"/>
       <c r="O260"/>
+      <c r="P260"/>
     </row>
     <row r="261">
       <c r="A261" t="n" s="22">
@@ -34746,13 +35008,13 @@
         <v>313</v>
       </c>
       <c r="F261" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="G261"/>
       <c r="H261"/>
       <c r="I261"/>
       <c r="J261" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K261" t="s">
         <v>1227</v>
@@ -34761,6 +35023,7 @@
       <c r="M261"/>
       <c r="N261"/>
       <c r="O261"/>
+      <c r="P261"/>
     </row>
     <row r="262">
       <c r="A262" t="n" s="22">
@@ -34777,13 +35040,13 @@
         <v>313</v>
       </c>
       <c r="F262" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G262"/>
       <c r="H262"/>
       <c r="I262"/>
       <c r="J262" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K262" t="s">
         <v>1227</v>
@@ -34792,6 +35055,7 @@
       <c r="M262"/>
       <c r="N262"/>
       <c r="O262"/>
+      <c r="P262"/>
     </row>
     <row r="263">
       <c r="A263" t="n" s="22">
@@ -34799,22 +35063,22 @@
       </c>
       <c r="B263"/>
       <c r="C263" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="D263" t="s">
-        <v>768</v>
+        <v>776</v>
       </c>
       <c r="E263" t="s">
-        <v>99</v>
+        <v>313</v>
       </c>
       <c r="F263" t="s">
-        <v>433</v>
+        <v>670</v>
       </c>
       <c r="G263"/>
       <c r="H263"/>
       <c r="I263"/>
       <c r="J263" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K263" t="s">
         <v>1227</v>
@@ -34823,6 +35087,7 @@
       <c r="M263"/>
       <c r="N263"/>
       <c r="O263"/>
+      <c r="P263"/>
     </row>
     <row r="264">
       <c r="A264" t="n" s="22">
@@ -34833,7 +35098,7 @@
         <v>98</v>
       </c>
       <c r="D264" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="E264" t="s">
         <v>99</v>
@@ -34845,7 +35110,7 @@
       <c r="H264"/>
       <c r="I264"/>
       <c r="J264" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K264" t="s">
         <v>1227</v>
@@ -34854,29 +35119,30 @@
       <c r="M264"/>
       <c r="N264"/>
       <c r="O264"/>
+      <c r="P264"/>
     </row>
     <row r="265">
       <c r="A265" t="n" s="22">
-        <v>43836.0</v>
+        <v>43101.0</v>
       </c>
       <c r="B265"/>
       <c r="C265" t="s">
-        <v>63</v>
+        <v>98</v>
       </c>
       <c r="D265" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="E265" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
       <c r="F265" t="s">
-        <v>68</v>
+        <v>433</v>
       </c>
       <c r="G265"/>
       <c r="H265"/>
       <c r="I265"/>
       <c r="J265" t="n">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="K265" t="s">
         <v>1227</v>
@@ -34885,6 +35151,7 @@
       <c r="M265"/>
       <c r="N265"/>
       <c r="O265"/>
+      <c r="P265"/>
     </row>
     <row r="266">
       <c r="A266" t="n" s="22">
@@ -34901,13 +35168,13 @@
         <v>73</v>
       </c>
       <c r="F266" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G266"/>
       <c r="H266"/>
       <c r="I266"/>
       <c r="J266" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K266" t="s">
         <v>1227</v>
@@ -34916,6 +35183,7 @@
       <c r="M266"/>
       <c r="N266"/>
       <c r="O266"/>
+      <c r="P266"/>
     </row>
     <row r="267">
       <c r="A267" t="n" s="22">
@@ -34932,13 +35200,13 @@
         <v>73</v>
       </c>
       <c r="F267" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G267"/>
       <c r="H267"/>
       <c r="I267"/>
       <c r="J267" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K267" t="s">
         <v>1227</v>
@@ -34947,6 +35215,7 @@
       <c r="M267"/>
       <c r="N267"/>
       <c r="O267"/>
+      <c r="P267"/>
     </row>
     <row r="268">
       <c r="A268" t="n" s="22">
@@ -34963,13 +35232,13 @@
         <v>73</v>
       </c>
       <c r="F268" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G268"/>
       <c r="H268"/>
       <c r="I268"/>
       <c r="J268" t="n">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="K268" t="s">
         <v>1227</v>
@@ -34978,6 +35247,7 @@
       <c r="M268"/>
       <c r="N268"/>
       <c r="O268"/>
+      <c r="P268"/>
     </row>
     <row r="269">
       <c r="A269" t="n" s="22">
@@ -34991,16 +35261,16 @@
         <v>768</v>
       </c>
       <c r="E269" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F269" t="s">
-        <v>68</v>
+        <v>684</v>
       </c>
       <c r="G269"/>
       <c r="H269"/>
       <c r="I269"/>
       <c r="J269" t="n">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="K269" t="s">
         <v>1227</v>
@@ -35009,6 +35279,7 @@
       <c r="M269"/>
       <c r="N269"/>
       <c r="O269"/>
+      <c r="P269"/>
     </row>
     <row r="270">
       <c r="A270" t="n" s="22">
@@ -35025,13 +35296,13 @@
         <v>72</v>
       </c>
       <c r="F270" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G270"/>
       <c r="H270"/>
       <c r="I270"/>
       <c r="J270" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="K270" t="s">
         <v>1227</v>
@@ -35040,6 +35311,7 @@
       <c r="M270"/>
       <c r="N270"/>
       <c r="O270"/>
+      <c r="P270"/>
     </row>
     <row r="271">
       <c r="A271" t="n" s="22">
@@ -35056,13 +35328,13 @@
         <v>72</v>
       </c>
       <c r="F271" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G271"/>
       <c r="H271"/>
       <c r="I271"/>
       <c r="J271" t="n">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="K271" t="s">
         <v>1227</v>
@@ -35071,6 +35343,7 @@
       <c r="M271"/>
       <c r="N271"/>
       <c r="O271"/>
+      <c r="P271"/>
     </row>
     <row r="272">
       <c r="A272" t="n" s="22">
@@ -35087,13 +35360,13 @@
         <v>72</v>
       </c>
       <c r="F272" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G272"/>
       <c r="H272"/>
       <c r="I272"/>
       <c r="J272" t="n">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="K272" t="s">
         <v>1227</v>
@@ -35102,6 +35375,7 @@
       <c r="M272"/>
       <c r="N272"/>
       <c r="O272"/>
+      <c r="P272"/>
     </row>
     <row r="273">
       <c r="A273" t="n" s="22">
@@ -35112,19 +35386,19 @@
         <v>63</v>
       </c>
       <c r="D273" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="E273" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F273" t="s">
-        <v>68</v>
+        <v>684</v>
       </c>
       <c r="G273"/>
       <c r="H273"/>
       <c r="I273"/>
       <c r="J273" t="n">
-        <v>1.0</v>
+        <v>8.0</v>
       </c>
       <c r="K273" t="s">
         <v>1227</v>
@@ -35133,6 +35407,7 @@
       <c r="M273"/>
       <c r="N273"/>
       <c r="O273"/>
+      <c r="P273"/>
     </row>
     <row r="274">
       <c r="A274" t="n" s="22">
@@ -35149,13 +35424,13 @@
         <v>73</v>
       </c>
       <c r="F274" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G274"/>
       <c r="H274"/>
       <c r="I274"/>
       <c r="J274" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K274" t="s">
         <v>1227</v>
@@ -35164,6 +35439,7 @@
       <c r="M274"/>
       <c r="N274"/>
       <c r="O274"/>
+      <c r="P274"/>
     </row>
     <row r="275">
       <c r="A275" t="n" s="22">
@@ -35180,13 +35456,13 @@
         <v>73</v>
       </c>
       <c r="F275" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G275"/>
       <c r="H275"/>
       <c r="I275"/>
       <c r="J275" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K275" t="s">
         <v>1227</v>
@@ -35195,6 +35471,7 @@
       <c r="M275"/>
       <c r="N275"/>
       <c r="O275"/>
+      <c r="P275"/>
     </row>
     <row r="276">
       <c r="A276" t="n" s="22">
@@ -35211,13 +35488,13 @@
         <v>73</v>
       </c>
       <c r="F276" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G276"/>
       <c r="H276"/>
       <c r="I276"/>
       <c r="J276" t="n">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="K276" t="s">
         <v>1227</v>
@@ -35226,6 +35503,7 @@
       <c r="M276"/>
       <c r="N276"/>
       <c r="O276"/>
+      <c r="P276"/>
     </row>
     <row r="277">
       <c r="A277" t="n" s="22">
@@ -35239,16 +35517,16 @@
         <v>770</v>
       </c>
       <c r="E277" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F277" t="s">
-        <v>68</v>
+        <v>684</v>
       </c>
       <c r="G277"/>
       <c r="H277"/>
       <c r="I277"/>
       <c r="J277" t="n">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="K277" t="s">
         <v>1227</v>
@@ -35257,6 +35535,7 @@
       <c r="M277"/>
       <c r="N277"/>
       <c r="O277"/>
+      <c r="P277"/>
     </row>
     <row r="278">
       <c r="A278" t="n" s="22">
@@ -35273,13 +35552,13 @@
         <v>72</v>
       </c>
       <c r="F278" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G278"/>
       <c r="H278"/>
       <c r="I278"/>
       <c r="J278" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="K278" t="s">
         <v>1227</v>
@@ -35288,6 +35567,7 @@
       <c r="M278"/>
       <c r="N278"/>
       <c r="O278"/>
+      <c r="P278"/>
     </row>
     <row r="279">
       <c r="A279" t="n" s="22">
@@ -35304,13 +35584,13 @@
         <v>72</v>
       </c>
       <c r="F279" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G279"/>
       <c r="H279"/>
       <c r="I279"/>
       <c r="J279" t="n">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="K279" t="s">
         <v>1227</v>
@@ -35319,6 +35599,7 @@
       <c r="M279"/>
       <c r="N279"/>
       <c r="O279"/>
+      <c r="P279"/>
     </row>
     <row r="280">
       <c r="A280" t="n" s="22">
@@ -35335,13 +35616,13 @@
         <v>72</v>
       </c>
       <c r="F280" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G280"/>
       <c r="H280"/>
       <c r="I280"/>
       <c r="J280" t="n">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="K280" t="s">
         <v>1227</v>
@@ -35350,6 +35631,7 @@
       <c r="M280"/>
       <c r="N280"/>
       <c r="O280"/>
+      <c r="P280"/>
     </row>
     <row r="281">
       <c r="A281" t="n" s="22">
@@ -35363,16 +35645,16 @@
         <v>770</v>
       </c>
       <c r="E281" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F281" t="s">
-        <v>68</v>
+        <v>684</v>
       </c>
       <c r="G281"/>
       <c r="H281"/>
       <c r="I281"/>
       <c r="J281" t="n">
-        <v>5.0</v>
+        <v>8.0</v>
       </c>
       <c r="K281" t="s">
         <v>1227</v>
@@ -35381,6 +35663,7 @@
       <c r="M281"/>
       <c r="N281"/>
       <c r="O281"/>
+      <c r="P281"/>
     </row>
     <row r="282">
       <c r="A282" t="n" s="22">
@@ -35397,13 +35680,13 @@
         <v>74</v>
       </c>
       <c r="F282" t="s">
-        <v>665</v>
+        <v>68</v>
       </c>
       <c r="G282"/>
       <c r="H282"/>
       <c r="I282"/>
       <c r="J282" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="K282" t="s">
         <v>1227</v>
@@ -35412,6 +35695,7 @@
       <c r="M282"/>
       <c r="N282"/>
       <c r="O282"/>
+      <c r="P282"/>
     </row>
     <row r="283">
       <c r="A283" t="n" s="22">
@@ -35428,13 +35712,13 @@
         <v>74</v>
       </c>
       <c r="F283" t="s">
-        <v>70</v>
+        <v>665</v>
       </c>
       <c r="G283"/>
       <c r="H283"/>
       <c r="I283"/>
       <c r="J283" t="n">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="K283" t="s">
         <v>1227</v>
@@ -35443,6 +35727,7 @@
       <c r="M283"/>
       <c r="N283"/>
       <c r="O283"/>
+      <c r="P283"/>
     </row>
     <row r="284">
       <c r="A284" t="n" s="22">
@@ -35459,13 +35744,13 @@
         <v>74</v>
       </c>
       <c r="F284" t="s">
-        <v>684</v>
+        <v>70</v>
       </c>
       <c r="G284"/>
       <c r="H284"/>
       <c r="I284"/>
       <c r="J284" t="n">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="K284" t="s">
         <v>1227</v>
@@ -35474,6 +35759,39 @@
       <c r="M284"/>
       <c r="N284"/>
       <c r="O284"/>
+      <c r="P284"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="n" s="22">
+        <v>43836.0</v>
+      </c>
+      <c r="B285"/>
+      <c r="C285" t="s">
+        <v>63</v>
+      </c>
+      <c r="D285" t="s">
+        <v>770</v>
+      </c>
+      <c r="E285" t="s">
+        <v>74</v>
+      </c>
+      <c r="F285" t="s">
+        <v>684</v>
+      </c>
+      <c r="G285"/>
+      <c r="H285"/>
+      <c r="I285"/>
+      <c r="J285" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="K285" t="s">
+        <v>1227</v>
+      </c>
+      <c r="L285"/>
+      <c r="M285"/>
+      <c r="N285"/>
+      <c r="O285"/>
+      <c r="P285"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>